<commit_message>
6a basis note: cite published Hirasawa papers only
</commit_message>
<xml_diff>
--- a/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
+++ b/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8890654-31B8-B64D-840B-1617218D5D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66CEE3D-ED82-2D4D-A132-7B7726D4A59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1280" yWindow="660" windowWidth="23100" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1280" yWindow="660" windowWidth="23100" windowHeight="21680" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2596,9 +2596,6 @@
     <t>https://doi.org/10.5194/egusphere-2026-5460</t>
   </si>
   <si>
-    <t>Basis conversion: CESM2/E3SMv2 emit 90 nm, UKESM1 172 nm (Hirasawa 2026, J. Climate). Restate tonnages at our 150 nm by (d_ours/d_model)^3 x (model CCN fraction / our CCN fraction), so we match cloud droplets, not raw particle counts (Hirasawa, pers. comm. 9/21/2026; CCN fractions from Hirasawa 2026 preprint, Table 1). Then gross up for plume survival; ESMs emit diffuse fluxes, ours is a point source.  Assumes (1) forcing is mostly cloud forcing, roughly true for CESM2, and (2) our 150 nm and the models' 90/172 nm particles stay airborne with an equally long lifetime.</t>
-  </si>
-  <si>
     <t>Note: Not accounting for direct aerosol forcing scales with salt mass, not droplets; significant above ~50 Tg/yr, dominant above ~200 Tg/yr.</t>
   </si>
   <si>
@@ -2990,6 +2987,9 @@
   </si>
   <si>
     <t>Tito Jankowski, tito.jankowski@renphil.org</t>
+  </si>
+  <si>
+    <t>Basis conversion: CESM2/E3SMv2 emit 90 nm, UKESM1 172 nm (Hirasawa 2026, J. Climate). Restate tonnages at our 150 nm by (d_ours/d_model)^3 x (model CCN fraction / our CCN fraction), so we match cloud droplets, not raw particle counts; CCN fractions from Hirasawa 2026 preprint, Table 1). Then gross up for plume survival; ESMs emit diffuse fluxes, ours is a point source.  Assumes (1) forcing is mostly cloud forcing, roughly true for CESM2, and (2) our 150 nm and the models' 90/172 nm particles stay airborne with an equally long lifetime.</t>
   </si>
 </sst>
 </file>
@@ -8529,7 +8529,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="344" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B1" s="344"/>
       <c r="C1" s="344"/>
@@ -8842,7 +8842,7 @@
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="173" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B31" s="173"/>
       <c r="C31" s="173"/>
@@ -9053,7 +9053,7 @@
         <v>0.49268352325187736</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="J6" s="118">
         <f t="shared" ref="J6:J17" si="1">MIN(E6,F6,G6)</f>
@@ -9372,7 +9372,7 @@
         <v>1.116935941917609</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J12" s="118">
         <f t="shared" si="1"/>
@@ -11058,7 +11058,7 @@
         <v>64</v>
       </c>
       <c r="D10" s="380" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E10" s="380"/>
       <c r="F10" s="380"/>
@@ -11133,7 +11133,7 @@
     </row>
     <row r="15" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="127" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B15" s="310">
         <f>'2. Cost Inputs'!B56/7</f>
@@ -11143,7 +11143,7 @@
         <v>830</v>
       </c>
       <c r="D15" s="380" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="E15" s="380"/>
       <c r="F15" s="380"/>
@@ -11217,7 +11217,7 @@
     </row>
     <row r="20" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="127" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B20" s="136">
         <f>SUM(B16:B19)+B22</f>
@@ -11227,7 +11227,7 @@
         <v>149</v>
       </c>
       <c r="D20" s="380" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="E20" s="380"/>
       <c r="F20" s="380"/>
@@ -11251,7 +11251,7 @@
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="127" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B22" s="135">
         <f>B14*B7*'2. Cost Inputs'!B58</f>
@@ -11261,7 +11261,7 @@
         <v>149</v>
       </c>
       <c r="D22" s="129" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="E22" s="137"/>
       <c r="F22" s="137"/>
@@ -11361,7 +11361,7 @@
         <v>149</v>
       </c>
       <c r="D28" s="381" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="E28" s="381"/>
       <c r="F28" s="381"/>
@@ -11378,7 +11378,7 @@
         <v>149</v>
       </c>
       <c r="D29" s="381" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="E29" s="381"/>
       <c r="F29" s="381"/>
@@ -11402,21 +11402,21 @@
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="127" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B31" s="138">
         <v>95</v>
       </c>
       <c r="C31" s="127" t="s">
+        <v>938</v>
+      </c>
+      <c r="D31" s="139" t="s">
         <v>939</v>
-      </c>
-      <c r="D31" s="139" t="s">
-        <v>940</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="127" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="B32" s="138">
         <v>0.2</v>
@@ -11425,7 +11425,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="139" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="E32" s="137"/>
       <c r="F32" s="137"/>
@@ -11496,7 +11496,7 @@
         <v>64</v>
       </c>
       <c r="D37" s="381" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="E37" s="381"/>
       <c r="F37" s="381"/>
@@ -11513,7 +11513,7 @@
         <v>149</v>
       </c>
       <c r="D38" s="381" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E38" s="381"/>
       <c r="F38" s="381"/>
@@ -11862,7 +11862,7 @@
         <v>2.2499999999999999E-2</v>
       </c>
       <c r="C19" s="238" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -11888,7 +11888,7 @@
         <v>1730000000000</v>
       </c>
       <c r="C23" s="238" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -11900,7 +11900,7 @@
         <v>0.71</v>
       </c>
       <c r="C24" s="238" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -11921,7 +11921,7 @@
         <v>0.9</v>
       </c>
       <c r="C26" s="238" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -11994,7 +11994,7 @@
         <v>512</v>
       </c>
       <c r="C34" s="238" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -12015,7 +12015,7 @@
         <v>21428.571428571428</v>
       </c>
       <c r="C36" s="238" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -12036,7 +12036,7 @@
         <v>200000</v>
       </c>
       <c r="C38" s="238" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -12075,7 +12075,7 @@
         <v>0.3</v>
       </c>
       <c r="C42" s="238" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.15">
@@ -12096,7 +12096,7 @@
         <v>180000</v>
       </c>
       <c r="C44" s="168" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.15">
@@ -12110,7 +12110,7 @@
     </row>
     <row r="46" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="247" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="B46" s="168">
         <f>B39+B40+B43+B45+B47</f>
@@ -12119,14 +12119,14 @@
     </row>
     <row r="47" spans="1:3" ht="91.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="240" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B47" s="168">
         <f>B31*B12*'2. Cost Inputs'!B58</f>
         <v>60903163.893253833</v>
       </c>
       <c r="C47" s="168" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.15">
@@ -12138,7 +12138,7 @@
         <v>22</v>
       </c>
       <c r="C48" s="168" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.15">
@@ -12150,7 +12150,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="C49" s="168" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -12162,7 +12162,7 @@
         <v>13300000000</v>
       </c>
       <c r="C50" s="238" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -12523,7 +12523,7 @@
         <v>475</v>
       </c>
       <c r="D14" s="380" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="E14" s="380"/>
       <c r="F14" s="380"/>
@@ -12584,7 +12584,7 @@
     </row>
     <row r="18" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="127" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B18" s="156">
         <f>SUM(B15:B17)+B20</f>
@@ -12618,7 +12618,7 @@
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="127" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B20" s="155">
         <f>B13*B9*'2. Cost Inputs'!B58</f>
@@ -12628,7 +12628,7 @@
         <v>149</v>
       </c>
       <c r="D20" s="129" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="E20" s="137"/>
       <c r="F20" s="137"/>
@@ -12729,7 +12729,7 @@
         <v>586</v>
       </c>
       <c r="D26" s="380" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="E26" s="380"/>
       <c r="F26" s="380"/>
@@ -12789,7 +12789,7 @@
     </row>
     <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="127" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B30" s="134">
         <v>0.44</v>
@@ -12798,7 +12798,7 @@
         <v>64</v>
       </c>
       <c r="D30" s="129" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -12887,7 +12887,7 @@
         <v>396</v>
       </c>
       <c r="D36" s="380" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E36" s="380"/>
       <c r="F36" s="380"/>
@@ -12989,7 +12989,7 @@
     </row>
     <row r="3" spans="1:8" ht="46" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="363" t="s">
-        <v>848</v>
+        <v>979</v>
       </c>
       <c r="B3" s="363"/>
       <c r="C3" s="363"/>
@@ -13477,7 +13477,7 @@
         <v>64</v>
       </c>
       <c r="D32" s="326" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G32" s="201"/>
       <c r="H32" s="339"/>
@@ -13667,7 +13667,7 @@
     </row>
     <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="168" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B39" s="287"/>
       <c r="C39" s="168"/>
@@ -13691,7 +13691,7 @@
     </row>
     <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="170" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B41" s="288"/>
       <c r="C41" s="289"/>
@@ -13723,7 +13723,7 @@
     </row>
     <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="274" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B43" s="342">
         <v>0.6</v>
@@ -13742,7 +13742,7 @@
     </row>
     <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="274" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B44" s="342">
         <v>3.3</v>
@@ -13761,7 +13761,7 @@
     </row>
     <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="274" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B45" s="342">
         <v>12</v>
@@ -14392,7 +14392,7 @@
         <v>664</v>
       </c>
       <c r="E16" s="193" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -14441,7 +14441,7 @@
         <v>660</v>
       </c>
       <c r="E20" s="363" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="F20" s="363"/>
       <c r="G20" s="363"/>
@@ -14464,7 +14464,7 @@
         <v>3630</v>
       </c>
       <c r="E21" s="363" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="F21" s="363"/>
       <c r="G21" s="363"/>
@@ -14487,7 +14487,7 @@
         <v>13200</v>
       </c>
       <c r="E22" s="363" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="F22" s="363"/>
       <c r="G22" s="363"/>
@@ -14610,7 +14610,7 @@
     </row>
     <row r="33" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="363" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B33" s="363"/>
       <c r="C33" s="363"/>
@@ -14670,7 +14670,7 @@
     </row>
     <row r="2" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="363" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B2" s="363"/>
       <c r="C2" s="363"/>
@@ -14721,7 +14721,7 @@
     </row>
     <row r="6" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="294" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B6" s="317">
         <f>'3b. Outputs - Ship Piggyback'!C32</f>
@@ -14731,7 +14731,7 @@
         <v>367</v>
       </c>
       <c r="D6" s="394" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="E6" s="394"/>
       <c r="F6" s="394"/>
@@ -15001,7 +15001,7 @@
       </c>
       <c r="D25" s="286"/>
       <c r="E25" s="321" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="G25" s="193"/>
       <c r="H25" s="168"/>
@@ -15069,7 +15069,7 @@
         <v>660</v>
       </c>
       <c r="E29" s="395" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="F29" s="395"/>
       <c r="G29" s="395"/>
@@ -15092,7 +15092,7 @@
         <v>3630</v>
       </c>
       <c r="E30" s="395" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="F30" s="395"/>
       <c r="G30" s="395"/>
@@ -15115,7 +15115,7 @@
         <v>13200</v>
       </c>
       <c r="E31" s="395" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="F31" s="395"/>
       <c r="G31" s="395"/>
@@ -15314,7 +15314,7 @@
     </row>
     <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="304" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B47" s="310">
         <f>'3b. Outputs - Ship Piggyback'!B43</f>
@@ -15324,12 +15324,12 @@
         <v>687</v>
       </c>
       <c r="D47" s="203" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="304" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B48" s="310">
         <f>'3b. Outputs - Ship Piggyback'!B41*24*'3b. Outputs - Ship Piggyback'!B16*B50/1000</f>
@@ -15341,7 +15341,7 @@
     </row>
     <row r="49" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="363" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B49" s="363"/>
       <c r="C49" s="363"/>
@@ -15352,16 +15352,16 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A50" s="304" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B50" s="327">
         <v>0.2</v>
       </c>
       <c r="C50" s="304" t="s">
+        <v>967</v>
+      </c>
+      <c r="D50" s="203" t="s">
         <v>968</v>
-      </c>
-      <c r="D50" s="203" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -15388,7 +15388,7 @@
     </row>
     <row r="53" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="363" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B53" s="363"/>
       <c r="C53" s="363"/>
@@ -15399,7 +15399,7 @@
     </row>
     <row r="54" spans="1:7" ht="91" x14ac:dyDescent="0.15">
       <c r="A54" s="304" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B54" s="327">
         <f>ROUND(B52*D54,0)</f>
@@ -15412,7 +15412,7 @@
         <v>0.85</v>
       </c>
       <c r="E54" s="203" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -15426,7 +15426,7 @@
         <v>537</v>
       </c>
       <c r="D55" s="234" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="E55" s="234" t="str">
         <f>"Cost at tab-1 power, "&amp;TEXT($B$6,"$#,##0")&amp;"/t ($B/yr)"</f>
@@ -15524,7 +15524,7 @@
     </row>
     <row r="61" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="393" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B61" s="393"/>
       <c r="C61" s="393"/>
@@ -15535,7 +15535,7 @@
     </row>
     <row r="62" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="363" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B62" s="363"/>
       <c r="C62" s="363"/>
@@ -15667,7 +15667,7 @@
         <v>702</v>
       </c>
       <c r="C3" s="316" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="D3" s="316" t="s">
         <v>703</v>
@@ -15681,7 +15681,7 @@
         <v>705</v>
       </c>
       <c r="C4" s="316" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="D4" s="316" t="s">
         <v>706</v>
@@ -15709,7 +15709,7 @@
         <v>712</v>
       </c>
       <c r="C6" s="316" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="D6" s="316" t="s">
         <v>713</v>
@@ -15723,7 +15723,7 @@
         <v>715</v>
       </c>
       <c r="C7" s="316" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="D7" s="316" t="s">
         <v>716</v>
@@ -15737,7 +15737,7 @@
         <v>718</v>
       </c>
       <c r="C8" s="316" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="D8" s="316" t="s">
         <v>719</v>
@@ -15751,7 +15751,7 @@
         <v>721</v>
       </c>
       <c r="C9" s="316" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="D9" s="316" t="s">
         <v>722</v>
@@ -15765,7 +15765,7 @@
         <v>724</v>
       </c>
       <c r="C10" s="316" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="D10" s="316" t="s">
         <v>725</v>
@@ -15793,7 +15793,7 @@
         <v>730</v>
       </c>
       <c r="C12" s="316" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="D12" s="316" t="s">
         <v>731</v>
@@ -15807,7 +15807,7 @@
         <v>733</v>
       </c>
       <c r="C13" s="316" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D13" s="316" t="s">
         <v>734</v>
@@ -15821,7 +15821,7 @@
         <v>846</v>
       </c>
       <c r="C14" s="316" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D14" s="316" t="s">
         <v>847</v>
@@ -15879,7 +15879,7 @@
         <v>746</v>
       </c>
       <c r="C19" s="316" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D19" s="316" t="s">
         <v>758</v>
@@ -15907,7 +15907,7 @@
         <v>751</v>
       </c>
       <c r="C21" s="316" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="D21" s="316" t="s">
         <v>760</v>
@@ -15937,7 +15937,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="166" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B1" s="179"/>
       <c r="C1" s="179"/>
@@ -16032,7 +16032,7 @@
         <v>24</v>
       </c>
       <c r="D10" s="208" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="E10" s="208" t="s">
         <v>789</v>
@@ -16123,7 +16123,7 @@
       <c r="E16" s="168"/>
       <c r="F16" s="168"/>
       <c r="G16" s="170" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.15">
@@ -16138,20 +16138,20 @@
         <v>35</v>
       </c>
       <c r="D17" s="208" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="E17" s="208" t="s">
         <v>790</v>
       </c>
       <c r="F17" s="168"/>
       <c r="G17" s="183" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="H17" s="194">
         <v>1</v>
       </c>
       <c r="I17" s="185" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
@@ -16169,7 +16169,7 @@
       <c r="E18" s="201"/>
       <c r="F18" s="168"/>
       <c r="G18" s="183" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="H18" s="194">
         <v>512</v>
@@ -16193,7 +16193,7 @@
       <c r="E19" s="201"/>
       <c r="F19" s="168"/>
       <c r="G19" s="183" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="H19" s="194">
         <v>51.2</v>
@@ -16219,7 +16219,7 @@
       <c r="E20" s="168"/>
       <c r="F20" s="168"/>
       <c r="G20" s="183" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -16294,16 +16294,16 @@
     </row>
     <row r="26" spans="1:9" ht="39" x14ac:dyDescent="0.15">
       <c r="A26" s="183" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B26" s="199">
         <v>0.6</v>
       </c>
       <c r="C26" s="185" t="s">
+        <v>889</v>
+      </c>
+      <c r="D26" s="208" t="s">
         <v>890</v>
-      </c>
-      <c r="D26" s="208" t="s">
-        <v>891</v>
       </c>
       <c r="E26" s="168"/>
       <c r="F26" s="168"/>
@@ -16497,7 +16497,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B1" s="209"/>
       <c r="C1" s="209"/>
@@ -16590,19 +16590,19 @@
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B8" s="20">
         <v>0.7</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>892</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>893</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>894</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>895</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16648,7 +16648,7 @@
     </row>
     <row r="12" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B12" s="16">
         <f>B13*'1. Technology Description'!B8*'1. Technology Description'!B9</f>
@@ -16659,7 +16659,7 @@
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="2" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="D13" s="21"/>
       <c r="E13" s="2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="F13" s="354"/>
       <c r="G13" s="354"/>
@@ -16692,10 +16692,10 @@
       </c>
       <c r="D14" s="21"/>
       <c r="E14" s="25" t="s">
+        <v>898</v>
+      </c>
+      <c r="F14" t="s">
         <v>899</v>
-      </c>
-      <c r="F14" t="s">
-        <v>900</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16932,7 +16932,7 @@
         <v>150000</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>107</v>
@@ -17026,7 +17026,7 @@
         <v>17</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.2">
@@ -17045,19 +17045,19 @@
         <v>100</v>
       </c>
       <c r="E40" s="33" t="s">
+        <v>901</v>
+      </c>
+      <c r="F40" s="33" t="s">
         <v>902</v>
       </c>
-      <c r="F40" s="33" t="s">
-        <v>903</v>
-      </c>
       <c r="G40" s="9" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="H40" s="31">
         <v>2</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -17081,7 +17081,7 @@
         <v>754</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="H41" s="31">
         <v>10</v>
@@ -17110,7 +17110,7 @@
         <v>756</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="H42" s="31">
         <v>100</v>
@@ -17137,7 +17137,7 @@
         <v>121</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H43" s="31">
         <v>1000</v>
@@ -17166,7 +17166,7 @@
         <v>757</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -17305,7 +17305,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="B56" s="31">
         <v>150000</v>
@@ -17314,7 +17314,7 @@
         <v>475</v>
       </c>
       <c r="D56" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E56" t="s">
         <v>832</v>
@@ -17322,7 +17322,7 @@
     </row>
     <row r="57" spans="1:6" ht="30" x14ac:dyDescent="0.2">
       <c r="A57" s="34" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B57" s="35">
         <f>(B40*D40+B41*D41+B42*D42)*(1+B49+B50+B52)+C51</f>
@@ -17332,12 +17332,12 @@
         <v>149</v>
       </c>
       <c r="D57" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="34" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B58" s="35">
         <f>B57*((B7*(1+B7)^B6)/((1+B7)^B6-1))/365</f>
@@ -17347,7 +17347,7 @@
         <v>830</v>
       </c>
       <c r="D58" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
   </sheetData>
@@ -18153,7 +18153,7 @@
     </row>
     <row r="26" spans="1:36" ht="104" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="B26" s="20">
         <v>0.9</v>
@@ -18162,7 +18162,7 @@
         <v>64</v>
       </c>
       <c r="E26" s="45" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="27" spans="1:36" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -18332,7 +18332,7 @@
         <v>8098.2326793128714</v>
       </c>
       <c r="E37" s="45" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="38" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -19069,7 +19069,7 @@
         <v>230</v>
       </c>
       <c r="F54" s="216" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="I54" s="217" t="s">
         <v>231</v>
@@ -21785,7 +21785,7 @@
     </row>
     <row r="2" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="363" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="B2" s="363"/>
       <c r="C2" s="363"/>
@@ -21882,7 +21882,7 @@
     </row>
     <row r="8" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="183" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B8" s="343">
         <f>'2. Cost Inputs'!D24</f>
@@ -21892,7 +21892,7 @@
         <v>240</v>
       </c>
       <c r="D8" s="364" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="E8" s="364" t="s">
         <v>279</v>
@@ -21942,7 +21942,7 @@
     </row>
     <row r="11" spans="1:7" ht="39" x14ac:dyDescent="0.15">
       <c r="A11" s="183" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="B11" s="221">
         <v>80000</v>
@@ -21951,7 +21951,7 @@
         <v>233</v>
       </c>
       <c r="D11" s="222" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -22140,7 +22140,7 @@
         <v>9100.3503524114603</v>
       </c>
       <c r="D27" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -22253,12 +22253,12 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A40" s="170" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="182" x14ac:dyDescent="0.15">
       <c r="A41" s="183" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B41" s="221">
         <v>4500</v>
@@ -22267,12 +22267,12 @@
         <v>117</v>
       </c>
       <c r="D41" s="222" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="39" x14ac:dyDescent="0.15">
       <c r="A42" s="183" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B42" s="231">
         <f>B41*1000/'1. Technology Description'!B17</f>
@@ -22282,12 +22282,12 @@
         <v>79</v>
       </c>
       <c r="D42" s="222" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="52" x14ac:dyDescent="0.15">
       <c r="A43" s="183" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B43" s="231">
         <f>($B$13+$B$14)*$B$42*'2. Cost Inputs'!$B$11</f>
@@ -22297,7 +22297,7 @@
         <v>76</v>
       </c>
       <c r="D43" s="222" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
   </sheetData>
@@ -22689,7 +22689,7 @@
         <v>4550.1751762057302</v>
       </c>
       <c r="D28" s="364" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="E28" s="364"/>
       <c r="F28" s="364"/>
@@ -23621,7 +23621,7 @@
     </row>
     <row r="13" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="97" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B13" s="20">
         <v>0.43</v>
@@ -23630,7 +23630,7 @@
         <v>64</v>
       </c>
       <c r="D13" s="369" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E13" s="369"/>
       <c r="F13" s="369"/>

</xml_diff>

<commit_message>
feat(workbook): annotate Tito's draft in place; add Survey, Summary, Sources tabs
Literature notes in an adjacent column (values unchanged), plus three
added tabs. Round-trip: 1246 formulas, 3 data validations, 2 charts, styles preserved.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118o5nFrXyN5L8uonKyjVV1
</commit_message>
<xml_diff>
--- a/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
+++ b/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
@@ -25,6 +25,9 @@
     <sheet name="6b. Benefit - Global - Vessel" sheetId="14" r:id="rId15"/>
     <sheet name="6c. Benefit - Global Piggyback" sheetId="15" r:id="rId16"/>
     <sheet name="References" sheetId="17" r:id="rId17"/>
+    <sheet name="Survey (added by precis)" sheetId="19" r:id="rId101"/>
+    <sheet name="Summary (added by precis)" sheetId="20" r:id="rId102"/>
+    <sheet name="Sources (added by precis)" sheetId="21" r:id="rId103"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -3017,7 +3020,7 @@
     <numFmt numFmtId="180" formatCode="\$#,##0.0"/>
     <numFmt numFmtId="181" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="57" x14ac:knownFonts="1">
+  <fonts count="62" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3405,8 +3408,36 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF375623"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3470,6 +3501,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF8EFA00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3619,7 +3668,7 @@
     <xf numFmtId="44" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="397">
+  <cellXfs count="404">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4556,6 +4605,27 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -12949,7 +13019,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="40" style="167" customWidth="1"/>
@@ -12962,7 +13032,9 @@
     <col min="8" max="8" width="17.83203125" style="167" customWidth="1"/>
     <col min="9" max="9" width="20" style="167" customWidth="1"/>
     <col min="10" max="10" width="33.5" style="167" customWidth="1"/>
-    <col min="11" max="16384" width="8.6640625" style="167"/>
+    <col min="11" max="13" width="8.6640625" style="167"/>
+    <col min="14" max="14" width="120" style="167" customWidth="1"/>
+    <col min="15" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
@@ -13020,7 +13092,7 @@
       <c r="F5" s="363"/>
       <c r="G5" s="363"/>
     </row>
-    <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="111" t="s">
         <v>614</v>
       </c>
@@ -13040,6 +13112,11 @@
       <c r="G6" s="111" t="s">
         <v>268</v>
       </c>
+      <c r="N6" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="270" t="s">
@@ -13106,7 +13183,7 @@
       </c>
       <c r="H9" s="387"/>
     </row>
-    <row r="10" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="270" t="s">
         <v>626</v>
       </c>
@@ -13127,6 +13204,11 @@
         <v>627</v>
       </c>
       <c r="H10" s="387"/>
+      <c r="N10" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFLICT: these K-per-Tg/yr values come from Hirasawa 2026 (https://doi.org/10.1175/JCLI-D-25-0337.1), not checked (full text unavailable). The preprint (https://doi.org/10.5194/egusphere-2026-5460) finds emissions for -2 W/m2 span 7-93 Tg/yr across nine models (13x); the workbook spread is 31x (0.236 vs 0.00754).</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="270" t="s">
@@ -13212,7 +13294,7 @@
       <c r="F15" s="363"/>
       <c r="G15" s="363"/>
     </row>
-    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="274" t="s">
         <v>836</v>
       </c>
@@ -13233,6 +13315,11 @@
         <v>834</v>
       </c>
       <c r="H16" s="387"/>
+      <c r="N16" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: for the same 50% droplet-number increase, 9 ESMs give ERF -0.6 to -2.5 W/m2 (4.2x), median -1.9 (Stjern 2018, https://doi.org/10.5194/acp-18-621-2018).</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="274" t="s">
@@ -13466,7 +13553,7 @@
       </c>
       <c r="I31" s="390"/>
     </row>
-    <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="168" t="s">
         <v>653</v>
       </c>
@@ -13482,6 +13569,11 @@
       <c r="G32" s="201"/>
       <c r="H32" s="339"/>
       <c r="I32" s="339"/>
+      <c r="N32" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFLICT: no literature value for survival to cloud base; open gap (https://doi.org/10.3389/fmars.2025.1450175). See tab 5a B5.</t>
+        </is>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="111" t="s">
@@ -13721,7 +13813,7 @@
       <c r="H42" s="168"/>
       <c r="I42" s="168"/>
     </row>
-    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="274" t="s">
         <v>951</v>
       </c>
@@ -13739,8 +13831,13 @@
       </c>
       <c r="H43" s="168"/>
       <c r="I43" s="168"/>
-    </row>
-    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="N43" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: Nordhaus DICE-2016R (NBER w22933, no DOI checked); not checked against the paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="274" t="s">
         <v>952</v>
       </c>
@@ -13758,8 +13855,13 @@
       </c>
       <c r="H44" s="168"/>
       <c r="I44" s="168"/>
-    </row>
-    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="N44" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: Burke et al. 2015 (https://doi.org/10.1038/nature15725) reports a non-linear response, ~23% lower global income by 2100 unmitigated (secondary summary), not a per-degC rate; 3.3%/degC is the workbook's own conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="274" t="s">
         <v>953</v>
       </c>
@@ -13777,6 +13879,11 @@
       </c>
       <c r="H45" s="168"/>
       <c r="I45" s="168"/>
+      <c r="N45" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: Bilal &amp; Kanzig 2024 (NBER w32450) coefficient not verified. Kotz et al. 2024 (https://doi.org/10.1038/s41586-024-07219-0): 19% lower world income by 2050 (11-29%), a level not a per-degC rate; not checked.</t>
+        </is>
+      </c>
     </row>
     <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="168"/>
@@ -14173,7 +14280,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="38" style="167" customWidth="1"/>
@@ -14184,7 +14291,9 @@
     <col min="6" max="6" width="25.5" style="167" customWidth="1"/>
     <col min="7" max="7" width="46" style="167" customWidth="1"/>
     <col min="8" max="8" width="10" style="167" customWidth="1"/>
-    <col min="9" max="16384" width="8.83203125" style="167"/>
+    <col min="9" max="9" width="8.83203125" style="167"/>
+    <col min="10" max="10" width="120" style="167" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -14407,7 +14516,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="234" t="s">
         <v>667</v>
       </c>
@@ -14422,6 +14531,11 @@
       </c>
       <c r="E19" s="234" t="s">
         <v>415</v>
+      </c>
+      <c r="J19" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scale cross-check: damage per degC already contains storm damage. 2026 EU hail/storm insured losses were EUR 6.1B for two events (PERILS, https://www.perils.org/news), ~0.2% of the central $3,630B per K-year; do not add as a separate line. AMOC effect on this benefit is model-dependent (Hirasawa 2023 https://doi.org/10.1029/2023GL104314; Xie 2022 https://doi.org/10.5194/acp-22-4581-2022).</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.15">
@@ -14642,7 +14756,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="42" style="167" customWidth="1"/>
@@ -14653,7 +14767,9 @@
     <col min="6" max="6" width="22" style="167" customWidth="1"/>
     <col min="7" max="7" width="18" style="167" customWidth="1"/>
     <col min="8" max="8" width="10" style="167" customWidth="1"/>
-    <col min="9" max="16384" width="8.83203125" style="167"/>
+    <col min="9" max="9" width="8.83203125" style="167"/>
+    <col min="10" max="10" width="120" style="167" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -15033,7 +15149,7 @@
       <c r="G27" s="168"/>
       <c r="H27" s="168"/>
     </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="234" t="s">
         <v>667</v>
       </c>
@@ -15051,6 +15167,11 @@
       </c>
       <c r="G28" s="168"/>
       <c r="H28" s="168"/>
+      <c r="J28" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scale cross-check: damage per degC already contains storm damage. 2026 EU hail/storm insured losses were EUR 6.1B for two events (PERILS, https://www.perils.org/news), ~0.2% of the central $3,630B per K-year. See tab 6b note.</t>
+        </is>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="304" t="s">
@@ -15922,9 +16043,3085 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="A1:H62"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
+    <col min="7" max="7" width="70" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Survey of the state of the art on this workbook's inputs and outputs. Flags: stub, perplexity-only, hand-FX, unverified, no-source, verified (legend on the Summary tab). Empty value cells mean no source was found. Source handles are the precis knowledge-graph ids.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quantity</t>
+        </is>
+      </c>
+      <c r="B3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unit</t>
+        </is>
+      </c>
+      <c r="D3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Range</t>
+        </is>
+      </c>
+      <c r="E3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source handle</t>
+        </is>
+      </c>
+      <c r="F3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Citation</t>
+        </is>
+      </c>
+      <c r="G3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quote / locator</t>
+        </is>
+      </c>
+      <c r="H3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A. Spray / nozzle cost and rate</t>
+        </is>
+      </c>
+      <c r="B4" s="401"/>
+      <c r="C4" s="401"/>
+      <c r="D4" s="401"/>
+      <c r="E4" s="401"/>
+      <c r="F4" s="401"/>
+      <c r="G4" s="401"/>
+      <c r="H4" s="401"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nozzle particle production rate (best nozzle tested)</t>
+        </is>
+      </c>
+      <c r="B5" s="397">
+        <v>1730000000000.0</v>
+      </c>
+      <c r="C5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">particles/s per nozzle</t>
+        </is>
+      </c>
+      <c r="D5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">71% of particles within 30-1000 nm dry diameter</t>
+        </is>
+      </c>
+      <c r="E5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238582</t>
+        </is>
+      </c>
+      <c r="F5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"This nozzle produces an estimated 1.73×10^12 s -1 droplets from 0.41 mL s -1 filtered seawater (and 0.3 L s -1 of air) with 71% of those particles being within the assumed MCB effectiveness range of 30 to 1000 nm dry diameter."</t>
+        </is>
+      </c>
+      <c r="H5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seawater flow per nozzle</t>
+        </is>
+      </c>
+      <c r="B6" s="397">
+        <v>0.41</v>
+      </c>
+      <c r="C6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
+      </c>
+      <c r="D6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">air 0.3 L/s</t>
+        </is>
+      </c>
+      <c r="E6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238582</t>
+        </is>
+      </c>
+      <c r="F6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">same sentence as above</t>
+        </is>
+      </c>
+      <c r="H6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nozzles needed for 1e15 CCN/s (30-1000 nm)</t>
+        </is>
+      </c>
+      <c r="B7" s="397">
+        <v>814</v>
+      </c>
+      <c r="C7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nozzles</t>
+        </is>
+      </c>
+      <c r="D7" s="397"/>
+      <c r="E7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238583</t>
+        </is>
+      </c>
+      <c r="F7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"To reach a target CCN production rate of 10^15 s -1 within the 30- 1000nm size range would require 814 of this current effervescent nozzle."</t>
+        </is>
+      </c>
+      <c r="H7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spray-equipment power for 814 nozzles (compressor 410.7 kW + pump 6.7 kW)</t>
+        </is>
+      </c>
+      <c r="B8" s="397">
+        <v>417.4</v>
+      </c>
+      <c r="C8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kW</t>
+        </is>
+      </c>
+      <c r="D8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">compressor eff. 0.72, pump eff. 0.75, 15 MPa</t>
+        </is>
+      </c>
+      <c r="E8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238583</t>
+        </is>
+      </c>
+      <c r="F8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Combined this spraying equipment would require 417.4 kW to supply the 814 nozzles."</t>
+        </is>
+      </c>
+      <c r="H8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Power per nozzle (derived: 417.4 kW / 814)</t>
+        </is>
+      </c>
+      <c r="B9" s="397">
+        <v>0.513</v>
+      </c>
+      <c r="C9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kW per nozzle</t>
+        </is>
+      </c>
+      <c r="D9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook uses 512 W (tab 3a, tornado input C49)</t>
+        </is>
+      </c>
+      <c r="E9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238583</t>
+        </is>
+      </c>
+      <c r="F9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arithmetic on the two quoted figures above; matches the workbook's 512 W.</t>
+        </is>
+      </c>
+      <c r="H9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARIEL prototype: 100 nozzles power</t>
+        </is>
+      </c>
+      <c r="B10" s="397">
+        <v>55</v>
+      </c>
+      <c r="C10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kW (approx.)</t>
+        </is>
+      </c>
+      <c r="D10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">implies ~550 W per nozzle</t>
+        </is>
+      </c>
+      <c r="E10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238584</t>
+        </is>
+      </c>
+      <c r="F10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"a prototype of 100 nozzles requiring approximately 55 kW facilitated the initial outdoor tests"</t>
+        </is>
+      </c>
+      <c r="H10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry particle size of best nozzle (count median diameter)</t>
+        </is>
+      </c>
+      <c r="B11" s="397">
+        <v>49.5</v>
+      </c>
+      <c r="C11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nm</t>
+        </is>
+      </c>
+      <c r="D11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSD 2.01; ~94% of particles below 200 nm</t>
+        </is>
+      </c>
+      <c r="E11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238581</t>
+        </is>
+      </c>
+      <c r="F11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
+        </is>
+      </c>
+      <c r="G11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"had a CMD of 49.5 nm dry particle diameter and a GSD of 2.01". The workbook's design point is 150 nm (tab 6a B20); see Summary.</t>
+        </is>
+      </c>
+      <c r="H11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nozzle + manifold unit price</t>
+        </is>
+      </c>
+      <c r="B12" s="397">
+        <v>50</v>
+      </c>
+      <c r="C12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$/nozzle (MeeFog price as cited by the workbook)</t>
+        </is>
+      </c>
+      <c r="D12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook bracket $10-$1,000; base $100</t>
+        </is>
+      </c>
+      <c r="E12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513654 (RRAP CS-07 final report 2025, pp.31,35 per workbook); web:513652 (CS-06)</t>
+        </is>
+      </c>
+      <c r="F12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reef Restoration &amp; Adaptation Program CS-07 / CS-06 final reports 2025</t>
+        </is>
+      </c>
+      <c r="G12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value is the workbook's/strand's citation. PDF is cached but has no extracted text, so the figure could not be read in precis.</t>
+        </is>
+      </c>
+      <c r="H12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compression + generation capex</t>
+        </is>
+      </c>
+      <c r="B13" s="397"/>
+      <c r="C13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$/kW</t>
+        </is>
+      </c>
+      <c r="D13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook uses 1,500 $/kW</t>
+        </is>
+      </c>
+      <c r="E13" s="397"/>
+      <c r="F13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook cites a used 200 hp CNG compressor yard listing; not in precis</t>
+        </is>
+      </c>
+      <c r="G13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No source in the graph.</t>
+        </is>
+      </c>
+      <c r="H13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vessel purchase price (70-80 m PSV newbuild)</t>
+        </is>
+      </c>
+      <c r="B14" s="397"/>
+      <c r="C14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="D14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook uses $30M (22.5-56M)</t>
+        </is>
+      </c>
+      <c r="E14" s="397"/>
+      <c r="F14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook cites Clarksons via Riviera Maritime Media; not in precis</t>
+        </is>
+      </c>
+      <c r="G14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No source in the graph.</t>
+        </is>
+      </c>
+      <c r="H14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vessel fuel burn and price (16,000 L/d underway, $0.9/L), crew, charter</t>
+        </is>
+      </c>
+      <c r="B15" s="397"/>
+      <c r="C15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">various</t>
+        </is>
+      </c>
+      <c r="D15" s="397"/>
+      <c r="E15" s="397"/>
+      <c r="F15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook cites PSV spec sheets and assumptions; none in precis</t>
+        </is>
+      </c>
+      <c r="G15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No source in the graph.</t>
+        </is>
+      </c>
+      <c r="H15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B. Forcing per unit effort and climate-model spread</t>
+        </is>
+      </c>
+      <c r="B16" s="401"/>
+      <c r="C16" s="401"/>
+      <c r="D16" s="401"/>
+      <c r="E16" s="401"/>
+      <c r="F16" s="401"/>
+      <c r="G16" s="401"/>
+      <c r="H16" s="401"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spray vessels to offset CO2 doubling (Flettner design, Salter et al.)</t>
+        </is>
+      </c>
+      <c r="B17" s="397">
+        <v>1500</v>
+      </c>
+      <c r="C17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vessels</t>
+        </is>
+      </c>
+      <c r="D17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">each ~150 kW (wind-derived)</t>
+        </is>
+      </c>
+      <c r="E17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509685 / pc5154182</t>
+        </is>
+      </c>
+      <c r="F17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Latham et al. (2012), 'Marine cloud brightening'</t>
+        </is>
+      </c>
+      <c r="G17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"about 1500 spray vessels, each consuming about 150 kW (derived from the wind), would be required to produce the globally averaged negative forcing of −3.7 W m−2 required to balance carbon dioxide doubling."</t>
+        </is>
+      </c>
+      <c r="H17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Forcing target for those vessels</t>
+        </is>
+      </c>
+      <c r="B18" s="397">
+        <v>-3.7</v>
+      </c>
+      <c r="C18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W/m2 (global mean)</t>
+        </is>
+      </c>
+      <c r="D18" s="397"/>
+      <c r="E18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509685 / pc5154182</t>
+        </is>
+      </c>
+      <c r="F18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Latham et al. (2012)</t>
+        </is>
+      </c>
+      <c r="G18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">same sentence as above</t>
+        </is>
+      </c>
+      <c r="H18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ensemble effective radiative forcing, +50% CDNC in low marine clouds, 9 ESMs</t>
+        </is>
+      </c>
+      <c r="B19" s="397">
+        <v>-1.9</v>
+      </c>
+      <c r="C19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W/m2 (median)</t>
+        </is>
+      </c>
+      <c r="D19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-0.6 to -2.5</t>
+        </is>
+      </c>
+      <c r="E19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509690 / pc5153550</t>
+        </is>
+      </c>
+      <c r="F19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
+        </is>
+      </c>
+      <c r="G19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"The model ensemble median effective radiative forcing (ERF) amounts to −1.9 W m−2, with a substantial inter-model spread of −0.6 to −2.5 W m−2."</t>
+        </is>
+      </c>
+      <c r="H19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ensemble global cooling for that forcing (2020-2069 vs RCP4.5)</t>
+        </is>
+      </c>
+      <c r="B20" s="397">
+        <v>-0.96</v>
+      </c>
+      <c r="C20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K (median)</t>
+        </is>
+      </c>
+      <c r="D20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-0.17 to -1.21</t>
+        </is>
+      </c>
+      <c r="E20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509690 / pc5153551</t>
+        </is>
+      </c>
+      <c r="F20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
+        </is>
+      </c>
+      <c r="G20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"a median of (for years 2020–2069) −0.96 [−0.17 to −1.21] K relative to the RCP4.5 scenario"</t>
+        </is>
+      </c>
+      <c r="H20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sea-salt emission needed for -2 W/m2, lowest model</t>
+        </is>
+      </c>
+      <c r="B21" s="397">
+        <v>7</v>
+      </c>
+      <c r="C21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tg/yr</t>
+        </is>
+      </c>
+      <c r="D21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 to 93 Tg/yr across nine models (13x)</t>
+        </is>
+      </c>
+      <c r="E21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513649 / pc5238641</t>
+        </is>
+      </c>
+      <c r="F21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
+        </is>
+      </c>
+      <c r="G21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"iSSA mass emissions to get −2 Wm−2 ranging from 7 Tg yr−1 to 93 Tg yr−1 in models."</t>
+        </is>
+      </c>
+      <c r="H21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sea-salt emission needed for -2 W/m2, highest model</t>
+        </is>
+      </c>
+      <c r="B22" s="397">
+        <v>93</v>
+      </c>
+      <c r="C22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tg/yr</t>
+        </is>
+      </c>
+      <c r="D22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">see above</t>
+        </is>
+      </c>
+      <c r="E22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513649 / pc5238641</t>
+        </is>
+      </c>
+      <c r="F22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
+        </is>
+      </c>
+      <c r="G22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">same sentence as above</t>
+        </is>
+      </c>
+      <c r="H22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emitted median modal radius across ESMs</t>
+        </is>
+      </c>
+      <c r="B23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28.1 to 72.5</t>
+        </is>
+      </c>
+      <c r="C23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nm</t>
+        </is>
+      </c>
+      <c r="D23" s="397"/>
+      <c r="E23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513649 / pc5238641</t>
+        </is>
+      </c>
+      <c r="F23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
+        </is>
+      </c>
+      <c r="G23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"the ESMs use median modal radii ranging from 28.1nm to 72.5nm, resulting in major differences in CCN concentration."</t>
+        </is>
+      </c>
+      <c r="H23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global cooling efficiency, CESM2 (midlatitude)</t>
+        </is>
+      </c>
+      <c r="B24" s="397">
+        <v>0.236</v>
+      </c>
+      <c r="C24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K per Tg/yr</t>
+        </is>
+      </c>
+      <c r="D24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook tab 6a E10</t>
+        </is>
+      </c>
+      <c r="E24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513648</t>
+        </is>
+      </c>
+      <c r="F24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate, doi:10.1175/JCLI-D-25-0337.1</t>
+        </is>
+      </c>
+      <c r="G24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value as entered in the workbook. Paper is a stub in precis (0 blocks), so the number could not be read in the source.</t>
+        </is>
+      </c>
+      <c r="H24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global cooling efficiency, E3SMv2 (midlatitude)</t>
+        </is>
+      </c>
+      <c r="B25" s="397">
+        <v>0.0372</v>
+      </c>
+      <c r="C25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K per Tg/yr</t>
+        </is>
+      </c>
+      <c r="D25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook tab 6a E11</t>
+        </is>
+      </c>
+      <c r="E25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513648</t>
+        </is>
+      </c>
+      <c r="F25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate</t>
+        </is>
+      </c>
+      <c r="G25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">as above</t>
+        </is>
+      </c>
+      <c r="H25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global cooling efficiency, UKESM1.0 (midlatitude)</t>
+        </is>
+      </c>
+      <c r="B26" s="397">
+        <v>0.00754</v>
+      </c>
+      <c r="C26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K per Tg/yr</t>
+        </is>
+      </c>
+      <c r="D26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook tab 6a E12; CESM2/UKESM1 ratio = 31x</t>
+        </is>
+      </c>
+      <c r="E26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513648</t>
+        </is>
+      </c>
+      <c r="F26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate</t>
+        </is>
+      </c>
+      <c r="G26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">as above</t>
+        </is>
+      </c>
+      <c r="H26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fraction of emitted aerosol surviving to cloud base</t>
+        </is>
+      </c>
+      <c r="B27" s="397"/>
+      <c r="C27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fraction</t>
+        </is>
+      </c>
+      <c r="D27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook uses 0.3 (0.1-0.5)</t>
+        </is>
+      </c>
+      <c r="E27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510540 / pc5168648</t>
+        </is>
+      </c>
+      <c r="F27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hernandez-Jaramillo, Kelaher &amp; Harrison, 'A review of plume dispersion and measurement techniques applicable to marine cloud brightening'</t>
+        </is>
+      </c>
+      <c r="G27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The review gives no number. It lists as a priority gap: "estimations of the portion of MCB aerosol reaching cloud base."</t>
+        </is>
+      </c>
+      <c r="H27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface temperature sensitivity to forcing (local, reef)</t>
+        </is>
+      </c>
+      <c r="B28" s="397">
+        <v>0.0225</v>
+      </c>
+      <c r="C28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">degC per W/m2</t>
+        </is>
+      </c>
+      <c r="D28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook tab 5a</t>
+        </is>
+      </c>
+      <c r="E28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513655 (RRAP T14, Harrison et al. 2019)</t>
+        </is>
+      </c>
+      <c r="F28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison et al. (2019), RRAP T14 Environmental Modelling of Large-Scale SRM</t>
+        </is>
+      </c>
+      <c r="G28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value as entered in the workbook. PDF cached with no extracted text.</t>
+        </is>
+      </c>
+      <c r="H28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C. Side effects and AMOC</t>
+        </is>
+      </c>
+      <c r="B29" s="401"/>
+      <c r="C29" s="401"/>
+      <c r="D29" s="401"/>
+      <c r="E29" s="401"/>
+      <c r="F29" s="401"/>
+      <c r="G29" s="401"/>
+      <c r="H29" s="401"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global mean precipitation change under +50% CDNC</t>
+        </is>
+      </c>
+      <c r="B30" s="397">
+        <v>-2.35</v>
+      </c>
+      <c r="C30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% (median)</t>
+        </is>
+      </c>
+      <c r="D30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-0.57 to -2.96</t>
+        </is>
+      </c>
+      <c r="E30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509690 / pc5153551</t>
+        </is>
+      </c>
+      <c r="F30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
+        </is>
+      </c>
+      <c r="G30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"a weak but significant precipitation decrease of −2.35 [−0.57 to −2.96] % due to a colder climate, but at low latitudes there is a 1.19 % increase over land."</t>
+        </is>
+      </c>
+      <c r="H30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low-latitude land precipitation change under +50% CDNC</t>
+        </is>
+      </c>
+      <c r="B31" s="397">
+        <v>1.19</v>
+      </c>
+      <c r="C31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="D31" s="397"/>
+      <c r="E31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa509690 / pc5153551</t>
+        </is>
+      </c>
+      <c r="F31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
+        </is>
+      </c>
+      <c r="G31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">same sentence as above</t>
+        </is>
+      </c>
+      <c r="H31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC under regional MCB (3 subtropical oceans, CESM2)</t>
+        </is>
+      </c>
+      <c r="B32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">increase in AMOC index and N. Atlantic gyre mixing depth (magnitude not extracted)</t>
+        </is>
+      </c>
+      <c r="C32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qualitative</t>
+        </is>
+      </c>
+      <c r="D32" s="397"/>
+      <c r="E32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510467 / pc5166683</t>
+        </is>
+      </c>
+      <c r="F32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa, Hingmire, Singh, Rasch &amp; Mitra (2023), 'Effect of Regional Marine Cloud Brightening Interventions on Climate Tipping Elements', GRL, doi:10.1029/2023GL104314</t>
+        </is>
+      </c>
+      <c r="G32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"increased Atlantic meridional overturning circulation (AMOC) index and North Atlantic gyre mixing depth (Figures 3c and 3h), indicating reduced AMOC collapse risk."</t>
+        </is>
+      </c>
+      <c r="H32" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipping-element risk under regional MCB (overall)</t>
+        </is>
+      </c>
+      <c r="B33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reduced overall; some patterns worsen some elements</t>
+        </is>
+      </c>
+      <c r="C33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qualitative</t>
+        </is>
+      </c>
+      <c r="D33" s="397"/>
+      <c r="E33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510467 / pc5166639</t>
+        </is>
+      </c>
+      <c r="F33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. (2023), GRL</t>
+        </is>
+      </c>
+      <c r="G33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"MCB simulations generally show reduced tipping element risk overall, but certain MCB patterns may exacerbate some tipping element changes"</t>
+        </is>
+      </c>
+      <c r="H33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC under GeoMIP brightening of ocean regions (6 ESMs)</t>
+        </is>
+      </c>
+      <c r="B34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC decreases tied to reduced air-ocean temperature difference and reduced Sept Arctic sea ice; solar dimming more effective than MCB per unit TOA forcing</t>
+        </is>
+      </c>
+      <c r="C34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qualitative</t>
+        </is>
+      </c>
+      <c r="D34" s="397"/>
+      <c r="E34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510522 / pc5179359</t>
+        </is>
+      </c>
+      <c r="F34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xie, Moore, Zhao, Wolovick &amp; Muri (2022), 'Impacts of three types of solar geoengineering on the Atlantic Meridional Overturning Circulation', ACP (published 8 Apr 2022)</t>
+        </is>
+      </c>
+      <c r="G34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"solar dimming is more effective than either marine cloud brightening or stratospheric aerosol injection." Note: the MCB experiment mimics cloud brightening by prescribing ocean brightening, not aerosol microphysics.</t>
+        </is>
+      </c>
+      <c r="H34" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC under regional Arctic solar dimming (proxy, not MCB)</t>
+        </is>
+      </c>
+      <c r="B35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4x stronger local dimming needed to save summer sea ice; MOC reduction and Labrador Sea convection shutdown still possible</t>
+        </is>
+      </c>
+      <c r="C35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qualitative</t>
+        </is>
+      </c>
+      <c r="D35" s="397"/>
+      <c r="E35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510511 / pc5180602</t>
+        </is>
+      </c>
+      <c r="F35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tilmes, Jahn, Kay, Holland &amp; Lamarque (2014), 'Can regional climate engineering save the summer Arctic sea ice?', GRL, doi:10.1002/2013GL058731</t>
+        </is>
+      </c>
+      <c r="G35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Even with regional Arctic dimming, a reduction in the strength of the oceanic meridional overturning circulation and a shut down of Labrador Sea deep convection are possible."</t>
+        </is>
+      </c>
+      <c r="H35" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC baseline: weakening since ~1950</t>
+        </is>
+      </c>
+      <c r="B36" s="397">
+        <v>3</v>
+      </c>
+      <c r="C36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sv (+/- 1)</t>
+        </is>
+      </c>
+      <c r="D36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC currently 'weakest in over a millennium' per proxy records cited therein</t>
+        </is>
+      </c>
+      <c r="E36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510518 / pc5179664</t>
+        </is>
+      </c>
+      <c r="F36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">van Westen, Kliphuis &amp; Dijkstra (2024), 'Physics-based early warning signal shows that AMOC is on tipping course', Sci. Adv., doi:10.1126/sciadv.adk1189</t>
+        </is>
+      </c>
+      <c r="G36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"indicates that the AMOC weakened by 3 ± 1 Sv since about 1950."</t>
+        </is>
+      </c>
+      <c r="H36" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fisheries / marine ecosystem effect (magnitude)</t>
+        </is>
+      </c>
+      <c r="B37" s="397"/>
+      <c r="C37" s="397"/>
+      <c r="D37" s="397"/>
+      <c r="E37" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">td510496 (no linked papers)</t>
+        </is>
+      </c>
+      <c r="F37" s="397"/>
+      <c r="G37" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Side-effects strand has no ingested papers yet.</t>
+        </is>
+      </c>
+      <c r="H37" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salt deposition on land (magnitude)</t>
+        </is>
+      </c>
+      <c r="B38" s="397"/>
+      <c r="C38" s="397"/>
+      <c r="D38" s="397"/>
+      <c r="E38" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">td510496 (no linked papers)</t>
+        </is>
+      </c>
+      <c r="F38" s="397"/>
+      <c r="G38" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Side-effects strand has no ingested papers yet.</t>
+        </is>
+      </c>
+      <c r="H38" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dollar value of maintaining AMOC</t>
+        </is>
+      </c>
+      <c r="B39" s="397"/>
+      <c r="C39" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="D39" s="397"/>
+      <c r="E39" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">td510498</t>
+        </is>
+      </c>
+      <c r="F39" s="397"/>
+      <c r="G39" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No economic valuation found among the 20 linked AMOC papers read at title/abstract level.</t>
+        </is>
+      </c>
+      <c r="H39" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D. MCB cost estimates in the literature (Perplexity only; secondary, not primary)</t>
+        </is>
+      </c>
+      <c r="B40" s="401"/>
+      <c r="C40" s="401"/>
+      <c r="D40" s="401"/>
+      <c r="E40" s="401"/>
+      <c r="F40" s="401"/>
+      <c r="G40" s="401"/>
+      <c r="H40" s="401"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MCB deployment cost, general literature (origin of the '~$10B/yr' framing)</t>
+        </is>
+      </c>
+      <c r="B41" s="397">
+        <v>10</v>
+      </c>
+      <c r="C41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$B/yr</t>
+        </is>
+      </c>
+      <c r="D41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'poorly characterized'</t>
+        </is>
+      </c>
+      <c r="E41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558 [42] PMC6784395</t>
+        </is>
+      </c>
+      <c r="F41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer citing one review (PMC6784395); review text not read</t>
+        </is>
+      </c>
+      <c r="G41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"One review reports that MCB deployment costs are poorly characterized but might be around $10 billion per year."</t>
+        </is>
+      </c>
+      <c r="H41" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NASEM logistics estimate, Arctic MCB</t>
+        </is>
+      </c>
+      <c r="B42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 per week for 0.01 W/m2</t>
+        </is>
+      </c>
+      <c r="C42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$M/week per 0.01 W/m2</t>
+        </is>
+      </c>
+      <c r="D42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity annualises to ~$26B per W/m2-yr</t>
+        </is>
+      </c>
+      <c r="E42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558 [33]</t>
+        </is>
+      </c>
+      <c r="F42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer; underlying NASEM text not read</t>
+        </is>
+      </c>
+      <c r="G42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Approximately $5 million per week to produce 0.01 W/m² of forcing."</t>
+        </is>
+      </c>
+      <c r="H42" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regional Arctic MCB fleet</t>
+        </is>
+      </c>
+      <c r="B43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">500-1,000 vessels; capex up to GBP 40bn; ~GBP 10bn/yr running</t>
+        </is>
+      </c>
+      <c r="C43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mixed</t>
+        </is>
+      </c>
+      <c r="D43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">media/interview estimate</t>
+        </is>
+      </c>
+      <c r="E43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558 [33]</t>
+        </is>
+      </c>
+      <c r="F43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer; underlying source not read</t>
+        </is>
+      </c>
+      <c r="G43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"500–1,000 vessels, with capital cost up to £40bn and continuation costs around £10bn/year." Currency left as reported (GBP), not converted.</t>
+        </is>
+      </c>
+      <c r="H43" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Airborne MCB concept</t>
+        </is>
+      </c>
+      <c r="B44" s="397">
+        <v>40</v>
+      </c>
+      <c r="C44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$bn/yr</t>
+        </is>
+      </c>
+      <c r="D44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">autonomous-ship electricity alone ~$41bn/yr</t>
+        </is>
+      </c>
+      <c r="E44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558 [44]</t>
+        </is>
+      </c>
+      <c r="F44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer citing iopscience 10.1088/2515-7620/ad2f71; not read</t>
+        </is>
+      </c>
+      <c r="G44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Estimated operational cost around $40bn/year"</t>
+        </is>
+      </c>
+      <c r="H44" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E. Damage per degree of warming (feeds the workbook's value-per-K)</t>
+        </is>
+      </c>
+      <c r="B45" s="401"/>
+      <c r="C45" s="401"/>
+      <c r="D45" s="401"/>
+      <c r="E45" s="401"/>
+      <c r="F45" s="401"/>
+      <c r="G45" s="401"/>
+      <c r="H45" s="401"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Damage, low (Nordhaus DICE-2016R)</t>
+        </is>
+      </c>
+      <c r="B46" s="397">
+        <v>0.6</v>
+      </c>
+      <c r="C46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% GDP per degC</t>
+        </is>
+      </c>
+      <c r="D46" s="397"/>
+      <c r="E46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no paper in precis)</t>
+        </is>
+      </c>
+      <c r="F46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nordhaus (2017), NBER w22933, as cited in workbook tab 6a G43</t>
+        </is>
+      </c>
+      <c r="G46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value as entered in the workbook. Source not ingested.</t>
+        </is>
+      </c>
+      <c r="H46" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Damage, central (Burke, Hsiang &amp; Miguel 2015)</t>
+        </is>
+      </c>
+      <c r="B47" s="397">
+        <v>3.3</v>
+      </c>
+      <c r="C47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% GDP per degC</t>
+        </is>
+      </c>
+      <c r="D47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workbook derives from ~23% at ~3.7 degC</t>
+        </is>
+      </c>
+      <c r="E47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510562</t>
+        </is>
+      </c>
+      <c r="F47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Burke, Hsiang &amp; Miguel (2015), Nature 527:235</t>
+        </is>
+      </c>
+      <c r="G47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value as entered in the workbook. Paper is a stub in precis (0 blocks); 3.3%/degC is the workbook's own conversion.</t>
+        </is>
+      </c>
+      <c r="H47" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Burke et al. 2015: global income loss by 2100, unmitigated</t>
+        </is>
+      </c>
+      <c r="B48" s="397">
+        <v>23</v>
+      </c>
+      <c r="C48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% lower income</t>
+        </is>
+      </c>
+      <c r="D48" s="397"/>
+      <c r="E48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558</t>
+        </is>
+      </c>
+      <c r="F48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer on Burke et al., doi:10.1038/nature15725</t>
+        </is>
+      </c>
+      <c r="G48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"approximately 23% lower global average income by 2100"</t>
+        </is>
+      </c>
+      <c r="H48" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Damage, high (Bilal &amp; Kanzig 2024)</t>
+        </is>
+      </c>
+      <c r="B49" s="397">
+        <v>12</v>
+      </c>
+      <c r="C49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% GDP per degC</t>
+        </is>
+      </c>
+      <c r="D49" s="397"/>
+      <c r="E49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no paper in precis)</t>
+        </is>
+      </c>
+      <c r="F49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bilal &amp; Kanzig (2024), NBER w32450, as cited in workbook tab 6a G45</t>
+        </is>
+      </c>
+      <c r="G49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value as entered in the workbook. Not ingested; Perplexity states it found no source exposing the paper's exact coefficient.</t>
+        </is>
+      </c>
+      <c r="H49" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub; unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kotz, Levermann &amp; Wenz 2024: world income loss by 2050</t>
+        </is>
+      </c>
+      <c r="B50" s="397">
+        <v>19</v>
+      </c>
+      <c r="C50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">% lower income</t>
+        </is>
+      </c>
+      <c r="D50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11-29% likely range</t>
+        </is>
+      </c>
+      <c r="E50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558</t>
+        </is>
+      </c>
+      <c r="F50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer on Kotz et al., Nature, doi:10.1038/s41586-024-07219-0</t>
+        </is>
+      </c>
+      <c r="G50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Projected 19% lower world income by 2050, with a likely range of 11–29%" (a level, not a per-degC coefficient; Perplexity notes it has been challenged).</t>
+        </is>
+      </c>
+      <c r="H50" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of hail losses that scales with temperature</t>
+        </is>
+      </c>
+      <c r="B51" s="397"/>
+      <c r="C51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="D51" s="397"/>
+      <c r="E51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558</t>
+        </is>
+      </c>
+      <c r="F51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perplexity answer</t>
+        </is>
+      </c>
+      <c r="G51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Hail ... Not sourced." Perplexity found no defensible figure.</t>
+        </is>
+      </c>
+      <c r="H51" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F. Benefit side: 2026 European severe convective storm (SCS) insured losses</t>
+        </is>
+      </c>
+      <c r="B52" s="401"/>
+      <c r="C52" s="401"/>
+      <c r="D52" s="401"/>
+      <c r="E52" s="401"/>
+      <c r="F52" s="401"/>
+      <c r="G52" s="401"/>
+      <c r="H52" s="401"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCS 'Cerry', 13-19 Jul 2026 (DE/FR/CH/IT): second estimate</t>
+        </is>
+      </c>
+      <c r="B53" s="397">
+        <v>2806.0</v>
+      </c>
+      <c r="C53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR m</t>
+        </is>
+      </c>
+      <c r="D53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">initial estimate 2,186; provisional</t>
+        </is>
+      </c>
+      <c r="E53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651</t>
+        </is>
+      </c>
+      <c r="F53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PERILS AG industry loss estimate (Zurich), released 20 Oct 2026, perils.org</t>
+        </is>
+      </c>
+      <c r="G53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"PERILS’ second estimate of the insurance market loss is EUR 2,806 million. This compares to the initial loss estimate of EUR 2,186 million."</t>
+        </is>
+      </c>
+      <c r="H53" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCS 'Raphaela', 26-28 Aug 2026 (FR/DE/CH/IT): first estimate</t>
+        </is>
+      </c>
+      <c r="B54" s="397">
+        <v>3296.0</v>
+      </c>
+      <c r="C54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR m</t>
+        </is>
+      </c>
+      <c r="D54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">provisional; large hail, wind, flash flood</t>
+        </is>
+      </c>
+      <c r="E54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513650</t>
+        </is>
+      </c>
+      <c r="F54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PERILS AG industry loss estimate (Zurich), released 19 Oct 2026, perils.org</t>
+        </is>
+      </c>
+      <c r="G54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"PERILS’ initial estimate of the insurance market loss is EUR 3,296 million. Losses were the result of large hail, high winds and flash flooding."</t>
+        </is>
+      </c>
+      <c r="H54" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum of the two PERILS estimates (derived)</t>
+        </is>
+      </c>
+      <c r="B55" s="397">
+        <v>6102.0</v>
+      </c>
+      <c r="C55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR m</t>
+        </is>
+      </c>
+      <c r="D55" s="397"/>
+      <c r="E55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651 + web:513650</t>
+        </is>
+      </c>
+      <c r="F55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arithmetic</t>
+        </is>
+      </c>
+      <c r="G55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2,806 + 3,296 = 6,102 (EUR 6.1B). Both estimates are provisional and PERILS says updates follow.</t>
+        </is>
+      </c>
+      <c r="H55" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Earlier vintage sum (Cerry initial + Raphaela)</t>
+        </is>
+      </c>
+      <c r="B56" s="397">
+        <v>5482.0</v>
+      </c>
+      <c r="C56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR m</t>
+        </is>
+      </c>
+      <c r="D56" s="397"/>
+      <c r="E56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651 + web:513650</t>
+        </is>
+      </c>
+      <c r="F56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arithmetic</t>
+        </is>
+      </c>
+      <c r="G56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2,186 + 3,296 = 5,482. This is the strand's earlier '~EUR 5.5B'; superseded by the 6,102 above.</t>
+        </is>
+      </c>
+      <c r="H56" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerry second estimate in USD</t>
+        </is>
+      </c>
+      <c r="B57" s="397">
+        <v>3208.7</v>
+      </c>
+      <c r="C57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m</t>
+        </is>
+      </c>
+      <c r="D57" s="397"/>
+      <c r="E57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651 + api.frankfurter.app</t>
+        </is>
+      </c>
+      <c r="F57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand conversion</t>
+        </is>
+      </c>
+      <c r="G57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2,806 x 1.1435. EUR/USD 1.1435, ECB reference rate via api.frankfurter.app, rate date 2026-07-17 (last ECB publication on/before event end 2026-07-19, a Sunday).</t>
+        </is>
+      </c>
+      <c r="H57" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Raphaela first estimate in USD</t>
+        </is>
+      </c>
+      <c r="B58" s="397">
+        <v>3837.5</v>
+      </c>
+      <c r="C58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m</t>
+        </is>
+      </c>
+      <c r="D58" s="397"/>
+      <c r="E58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513650 + api.frankfurter.app</t>
+        </is>
+      </c>
+      <c r="F58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand conversion</t>
+        </is>
+      </c>
+      <c r="G58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3,296 x 1.1643. EUR/USD 1.1643, ECB reference rate via api.frankfurter.app, rate date 2026-08-28 (event end date).</t>
+        </is>
+      </c>
+      <c r="H58" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum of the two events in USD (event-date rates)</t>
+        </is>
+      </c>
+      <c r="B59" s="397">
+        <v>7046.2</v>
+      </c>
+      <c r="C59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m</t>
+        </is>
+      </c>
+      <c r="D59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6843.4 at the release-date rate 1.1215 (ECB 2026-10-20)</t>
+        </is>
+      </c>
+      <c r="E59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651 + web:513650 + api.frankfurter.app</t>
+        </is>
+      </c>
+      <c r="F59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand conversion</t>
+        </is>
+      </c>
+      <c r="G59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3208.7 + 3837.5. Release-date sensitivity: 6,102 x 1.1215 = 6843.4.</t>
+        </is>
+      </c>
+      <c r="H59" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Europe SCS insured losses, 9M 2026 (Gallagher Re)</t>
+        </is>
+      </c>
+      <c r="B60" s="397">
+        <v>9000</v>
+      </c>
+      <c r="C60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m (at least)</t>
+        </is>
+      </c>
+      <c r="D60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes USD 3.8B for the late-August outbreak</t>
+        </is>
+      </c>
+      <c r="E60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513656</t>
+        </is>
+      </c>
+      <c r="F60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinsurance News, 21 Oct 2026, reporting Gallagher Re Q3 2026 Natural Catastrophe and Climate Report (primary report page web:513653 has no extractable text)</t>
+        </is>
+      </c>
+      <c r="G60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"In Europe, insured losses associated with severe convective storms reached at least USD $9 billion, according to Gallagher Re. This included USD $3.8 billion in losses resulting from an outbreak in late August." Secondary relay.</t>
+        </is>
+      </c>
+      <c r="H60" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gallagher late-August Europe SCS vs PERILS Raphaela converted</t>
+        </is>
+      </c>
+      <c r="B61" s="397">
+        <v>3800</v>
+      </c>
+      <c r="C61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m</t>
+        </is>
+      </c>
+      <c r="D61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PERILS Raphaela converted = 3837.5</t>
+        </is>
+      </c>
+      <c r="E61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513656 vs web:513650</t>
+        </is>
+      </c>
+      <c r="F61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cross-check</t>
+        </is>
+      </c>
+      <c r="G61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gallagher 3.8B USD against 3,296 EUR x 1.1643: consistent at 2 significant figures. Different insurer scopes.</t>
+        </is>
+      </c>
+      <c r="H61" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US SCS insured losses, 9M 2026 (context)</t>
+        </is>
+      </c>
+      <c r="B62" s="397">
+        <v>43000</v>
+      </c>
+      <c r="C62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USD m (at least)</t>
+        </is>
+      </c>
+      <c r="D62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">global insured nat cat: USD 92B</t>
+        </is>
+      </c>
+      <c r="E62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513656</t>
+        </is>
+      </c>
+      <c r="F62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinsurance News on Gallagher Re</t>
+        </is>
+      </c>
+      <c r="G62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"insured losses from these storms in the United States reached at least USD $43 billion by the end of the third quarter."</t>
+        </is>
+      </c>
+      <c r="H62" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A52:H52"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Reads the workbook's figures against the Survey tab. Workbook numbers were read from the file unchanged; no workbook formula or value was edited. Literature notes sit in an adjacent column on the tabs themselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="B3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook value</t>
+        </is>
+      </c>
+      <c r="C3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook location</t>
+        </is>
+      </c>
+      <c r="D3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey comparison</t>
+        </is>
+      </c>
+      <c r="E3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey handle</t>
+        </is>
+      </c>
+      <c r="F3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading</t>
+        </is>
+      </c>
+      <c r="G3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLUF: (1) The workbook contains no '~$10B/yr' figure; its cost anchors are $21.4M/yr per dedicated vessel, $9.3M/yr per piggyback ship and $175B-$18T/yr for 1 K of global cooling. (2) Its nozzle power (512 W) and output (1.73e12 particles/s) match the Harrison et al. 2025 paper held in precis, but the 150 nm design size is not what that nozzle makes (count median 49.5 nm). (3) Its tonnage-per-K spread (31x) comes from a J. Climate paper that is a stub in precis; the full-text preprint by the same group gives 13x for equal forcing. (4) The damage-per-K band (0.6/3.3/12 % of GDP) rests on sources with no text in precis. (5) The two 2026 EU storm events (about USD 7.0B insured, hand-converted) are 329 dedicated vessel-years or 761 piggyback ship-years of Tito's cost, and 0.04%-4.0% of his per-K annual cost; hail and AMOC bear on the benefit side only as a scale cross-check and a model-dependent caveat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The '~$10B/yr' framing</t>
+        </is>
+      </c>
+      <c r="B5" s="401"/>
+      <c r="C5" s="401"/>
+      <c r="D5" s="401"/>
+      <c r="E5" s="401"/>
+      <c r="F5" s="401"/>
+      <c r="G5" s="401"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'~$10B/yr' deployment cost</t>
+        </is>
+      </c>
+      <c r="B6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">does NOT appear</t>
+        </is>
+      </c>
+      <c r="C6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">searched all 17 tabs: no text match and no numeric cell between 9e9 and 1.1e10</t>
+        </is>
+      </c>
+      <c r="D6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The framing traces to a Perplexity summary of one review ('might be around $10 billion per year'), not to the workbook.</t>
+        </is>
+      </c>
+      <c r="E6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-reasoning:510558 [42]</t>
+        </is>
+      </c>
+      <c r="F6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nearest workbook number: one piggyback ship at $9.26M/yr (tab 3b), 1000x smaller. Per-K cost $175B-$18T/yr is 17x to 1,800x the $10B. Comparisons below use the workbook's own costs.</t>
+        </is>
+      </c>
+      <c r="G6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">perplexity-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Workbook cost figures against the survey</t>
+        </is>
+      </c>
+      <c r="B7" s="401"/>
+      <c r="C7" s="401"/>
+      <c r="D7" s="401"/>
+      <c r="E7" s="401"/>
+      <c r="F7" s="401"/>
+      <c r="G7" s="401"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Levelized cost, dedicated vessel</t>
+        </is>
+      </c>
+      <c r="B8" s="397">
+        <v>54048</v>
+      </c>
+      <c r="C8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3a C13 ($/t); annual $21,389,498 (3a B13)</t>
+        </is>
+      </c>
+      <c r="D8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No independent $/t exists in the survey. Inputs: nozzle power 513 W derived vs 512 W used, particle rate 1.73e12/s identical.</t>
+        </is>
+      </c>
+      <c r="E8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238582, pc5238583</t>
+        </is>
+      </c>
+      <c r="F8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Energy input confirmed by source. Vessel price, fuel, compressor $/kW, survival 0.3 have no source in precis. Nozzle price $50 cited to RRAP CS-07 (no text).</t>
+        </is>
+      </c>
+      <c r="G8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified; no-source; stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Levelized cost, piggyback (3b)</t>
+        </is>
+      </c>
+      <c r="B9" s="397">
+        <v>21674</v>
+      </c>
+      <c r="C9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 B7 ($/t); $9,259,922/yr (4 C7)</t>
+        </is>
+      </c>
+      <c r="D9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deck-slot rent $2M, technicians, 4.5 MW gensets: no survey source.</t>
+        </is>
+      </c>
+      <c r="E9" s="397"/>
+      <c r="F9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No source in precis for the scenario-specific lines.</t>
+        </is>
+      </c>
+      <c r="G9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Levelized cost, fixed platform (3c)</t>
+        </is>
+      </c>
+      <c r="B10" s="397">
+        <v>14633</v>
+      </c>
+      <c r="C10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 B8 ($/t); $5,791,171/yr (4 C8)</t>
+        </is>
+      </c>
+      <c r="D10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platform $3M, siting, mooring, shore power: no survey source.</t>
+        </is>
+      </c>
+      <c r="E10" s="397"/>
+      <c r="F10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+      <c r="G10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Levelized cost, stationary vessel (3d)</t>
+        </is>
+      </c>
+      <c r="B11" s="397">
+        <v>49341</v>
+      </c>
+      <c r="C11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 B9 ($/t); $19,526,858/yr (4 C9)</t>
+        </is>
+      </c>
+      <c r="D11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No survey source.</t>
+        </is>
+      </c>
+      <c r="E11" s="397"/>
+      <c r="F11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+      <c r="G11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Particle size at design point</t>
+        </is>
+      </c>
+      <c r="B12" s="397">
+        <v>150</v>
+      </c>
+      <c r="C12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a B20 (nm)</t>
+        </is>
+      </c>
+      <c r="D12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nozzle count median diameter 49.5 nm, GSD 2.01. ESMs emit 28.1-72.5 nm (preprint); workbook restates tonnage to 150 nm via (150/d)^3.</t>
+        </is>
+      </c>
+      <c r="E12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513647 / pc5238581; pa513649 / pc5238641</t>
+        </is>
+      </c>
+      <c r="F12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open question for Tito: how a nozzle with CMD 49.5 nm yields the 150 nm design basis (the cubic size correction in 6a F34:F37 moves tonnage by factors of 0.75-1.02 only).</t>
+        </is>
+      </c>
+      <c r="G12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Climate-model spread, K per Tg/yr (CESM2 / UKESM1)</t>
+        </is>
+      </c>
+      <c r="B13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31x (0.236 vs 0.00754)</t>
+        </is>
+      </c>
+      <c r="C13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a E10, E12</t>
+        </is>
+      </c>
+      <c r="D13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preprint, equal -2 W/m2: emissions 7-93 Tg/yr = 13x. GeoMIP G4cdnc ERF for the same CDNC change: -0.6 to -2.5 W/m2 = 4.2x.</t>
+        </is>
+      </c>
+      <c r="E13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa513649 / pc5238641; pa509690 / pc5153550</t>
+        </is>
+      </c>
+      <c r="F13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workbook spread is the J. Climate paper's (stub, cannot be checked). The two full-text sources give a smaller spread.</t>
+        </is>
+      </c>
+      <c r="G13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value of 1 K for a year, low</t>
+        </is>
+      </c>
+      <c r="B14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$660B</t>
+        </is>
+      </c>
+      <c r="C14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D20 (0.6% x $110T)</t>
+        </is>
+      </c>
+      <c r="D14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nordhaus DICE source not ingested.</t>
+        </is>
+      </c>
+      <c r="E14" s="397"/>
+      <c r="F14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value is arithmetic on a GDP share with no source text.</t>
+        </is>
+      </c>
+      <c r="G14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value of 1 K for a year, central</t>
+        </is>
+      </c>
+      <c r="B15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$3,630B</t>
+        </is>
+      </c>
+      <c r="C15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D21 (3.3% x $110T)</t>
+        </is>
+      </c>
+      <c r="D15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Burke 2015 is a stub; the 3.3%/degC is the workbook's conversion of ~23% at ~3.7 degC. Perplexity gives 23% by 2100 (not a per-degC rate).</t>
+        </is>
+      </c>
+      <c r="E15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510562; perplexity-reasoning:510558</t>
+        </is>
+      </c>
+      <c r="F15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Central case has no readable source in precis.</t>
+        </is>
+      </c>
+      <c r="G15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value of 1 K for a year, high</t>
+        </is>
+      </c>
+      <c r="B16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$13,200B</t>
+        </is>
+      </c>
+      <c r="C16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D22 (12% x $110T)</t>
+        </is>
+      </c>
+      <c r="D16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bilal &amp; Kanzig 2024 not ingested; Perplexity could not find the coefficient.</t>
+        </is>
+      </c>
+      <c r="E16" s="397"/>
+      <c r="F16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Treat as unverified.</t>
+        </is>
+      </c>
+      <c r="G16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub; unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCR, dedicated vessel, 4 model cases</t>
+        </is>
+      </c>
+      <c r="B17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.64 / 8.30 / 0.877 / 0.202</t>
+        </is>
+      </c>
+      <c r="C17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D29:D32 (CESM2, CESM2-Ghosh, E3SMv2, UKESM1); costs $0.78T / $0.44T / $4.14T / $17.97T per year</t>
+        </is>
+      </c>
+      <c r="D17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numerator is the central $3,630B (stub-sourced); denominator spread is the 31x tonnage spread (stub-sourced).</t>
+        </is>
+      </c>
+      <c r="E17" s="397"/>
+      <c r="F17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both halves of the ratio rest on sources not readable in precis. The 6b header says '$B/yr' but cells hold raw dollars.</t>
+        </is>
+      </c>
+      <c r="G17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCR, piggyback, 4 model cases</t>
+        </is>
+      </c>
+      <c r="B18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11.6 / 20.7 / 2.19 / 0.504</t>
+        </is>
+      </c>
+      <c r="C18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6c D38:D41; costs $0.31T / $0.18T / $1.66T / $7.21T per year</t>
+        </is>
+      </c>
+      <c r="D18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same as above.</t>
+        </is>
+      </c>
+      <c r="E18" s="397"/>
+      <c r="F18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same as above.</t>
+        </is>
+      </c>
+      <c r="G18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cooling from one dedicated vessel (consistency check)</t>
+        </is>
+      </c>
+      <c r="B19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.74e-05 K</t>
+        </is>
+      </c>
+      <c r="C19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">396 t/yr (3a B22) / 14.46 Mt/yr (6b D10, CESM2)</t>
+        </is>
+      </c>
+      <c r="D19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value at central damage = $99.4M against $21.4M cost = BCR 4.64, equal to 6b D29.</t>
+        </is>
+      </c>
+      <c r="E19" s="397"/>
+      <c r="F19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Internal arithmetic only; confirms 6b is consistent with 3a.</t>
+        </is>
+      </c>
+      <c r="G19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. 2026 EU storm losses against Tito's per-vessel and per-K costs (not against $10B)</t>
+        </is>
+      </c>
+      <c r="B20" s="401"/>
+      <c r="C20" s="401"/>
+      <c r="D20" s="401"/>
+      <c r="E20" s="401"/>
+      <c r="F20" s="401"/>
+      <c r="G20" s="401"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two EU events, insured, in USD</t>
+        </is>
+      </c>
+      <c r="B21" s="397">
+        <v>7046.2</v>
+      </c>
+      <c r="C21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">survey F (USD m)</t>
+        </is>
+      </c>
+      <c r="D21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PERILS EUR 2,806m + 3,296m = EUR 6,102m, converted at event-date ECB rates</t>
+        </is>
+      </c>
+      <c r="E21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651, web:513650, api.frankfurter.app</t>
+        </is>
+      </c>
+      <c r="F21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR/USD 1.1435, ECB reference rate via api.frankfurter.app, rate date 2026-07-17 (last ECB publication on/before event end 2026-07-19, a Sunday); EUR/USD 1.1643, ECB reference rate via api.frankfurter.app, rate date 2026-08-28 (event end date).</t>
+        </is>
+      </c>
+      <c r="G21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">... in dedicated vessel-years</t>
+        </is>
+      </c>
+      <c r="B22" s="397">
+        <v>329.4</v>
+      </c>
+      <c r="C22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vs 3a B13 $21,389,498/yr</t>
+        </is>
+      </c>
+      <c r="D22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">329.4 vessel-years; one vessel-year = 0.30% of the two events</t>
+        </is>
+      </c>
+      <c r="E22" s="397"/>
+      <c r="F22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Insured loss of two events divided by one vessel's annual levelized cost.</t>
+        </is>
+      </c>
+      <c r="G22" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">... in piggyback ship-years</t>
+        </is>
+      </c>
+      <c r="B23" s="397">
+        <v>760.9</v>
+      </c>
+      <c r="C23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vs 4 C7 $9,259,922/yr</t>
+        </is>
+      </c>
+      <c r="D23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">760.9 ship-years; one ship-year = 0.13% of the two events</t>
+        </is>
+      </c>
+      <c r="E23" s="397"/>
+      <c r="F23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+      <c r="G23" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">... as share of dedicated-vessel cost of 1 K (4 cases)</t>
+        </is>
+      </c>
+      <c r="B24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.902% / 1.61% / 0.17% / 0.0392%</t>
+        </is>
+      </c>
+      <c r="C24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b E10:E13</t>
+        </is>
+      </c>
+      <c r="D24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CESM2 / CESM2-Ghosh / E3SMv2 / UKESM1</t>
+        </is>
+      </c>
+      <c r="E24" s="397"/>
+      <c r="F24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two events alone pay 0.04%-0.9% of a year of 1 K cooling.</t>
+        </is>
+      </c>
+      <c r="G24" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">... as share of piggyback cost of 1 K (4 cases)</t>
+        </is>
+      </c>
+      <c r="B25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.25% / 4.02% / 0.425% / 0.0978%</t>
+        </is>
+      </c>
+      <c r="C25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6c E18:E21</t>
+        </is>
+      </c>
+      <c r="D25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CESM2 / CESM2-Ghosh / E3SMv2 / UKESM1</t>
+        </is>
+      </c>
+      <c r="E25" s="397"/>
+      <c r="F25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two events alone pay 0.1%-4.0% of a year of 1 K cooling.</t>
+        </is>
+      </c>
+      <c r="G25" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">... as share of the workbook's value of 1 K-yr (low/central/high)</t>
+        </is>
+      </c>
+      <c r="B26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.07% / 0.194% / 0.0534%</t>
+        </is>
+      </c>
+      <c r="C26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D20:D22</t>
+        </is>
+      </c>
+      <c r="D26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$660B / $3,630B / $13,200B</t>
+        </is>
+      </c>
+      <c r="E26" s="397"/>
+      <c r="F26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Insured storm losses are a small slice of the damage-function value.</t>
+        </is>
+      </c>
+      <c r="G26" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gallagher Re: Europe SCS 9M 2026, at least USD 9B</t>
+        </is>
+      </c>
+      <c r="B27" s="397">
+        <v>9000</v>
+      </c>
+      <c r="C27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">survey F (USD m)</t>
+        </is>
+      </c>
+      <c r="D27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">421 dedicated vessel-years; 972 piggyback ship-years</t>
+        </is>
+      </c>
+      <c r="E27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513656</t>
+        </is>
+      </c>
+      <c r="F27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole-year-to-date Europe, USD as reported (no conversion). Includes the late-August USD 3.8B outbreak, so it overlaps the PERILS sum; do not add them.</t>
+        </is>
+      </c>
+      <c r="G27" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limits of this comparison: two events in one season are not an annual loss; insured loss is below economic loss; PERILS estimates are provisional (updates follow); and no source in precis says how much of this hail loss 1 K of marine cloud brightening would avoid (Perplexity: share of hail loss that scales with temperature 'Not sourced'). The storm losses are therefore context for scale, not a benefit line to add to 6b/6c, and would partly overlap the damage-function value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Where hail and AMOC bear on what the workbook computes</t>
+        </is>
+      </c>
+      <c r="B29" s="401"/>
+      <c r="C29" s="401"/>
+      <c r="D29" s="401"/>
+      <c r="E29" s="401"/>
+      <c r="F29" s="401"/>
+      <c r="G29" s="401"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hail / severe convective storm insured loss vs the damage-function value</t>
+        </is>
+      </c>
+      <c r="B30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR 6,102m (about USD 7046m) for two 2026 events</t>
+        </is>
+      </c>
+      <c r="C30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b D20:D22 value of 1 K-yr</t>
+        </is>
+      </c>
+      <c r="D30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The workbook values cooling through GDP-wide damage per degC, which already contains storm damage. Two events are 0.194% of the central $3,630B/K-yr: a scale cross-check, not an extra line to add.</t>
+        </is>
+      </c>
+      <c r="E30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web:513651, web:513650</t>
+        </is>
+      </c>
+      <c r="F30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No source in precis gives the hail share of the damage function or the hail loss avoided per K.</t>
+        </is>
+      </c>
+      <c r="G30" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand-FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMOC</t>
+        </is>
+      </c>
+      <c r="B31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qualitative only</t>
+        </is>
+      </c>
+      <c r="C31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b/6c benefit side (value of cooling)</t>
+        </is>
+      </c>
+      <c r="D31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whether the cooling benefit includes reduced AMOC-collapse risk is model-dependent: CESM2 regional MCB raises the AMOC index (Hirasawa 2023); GeoMIP ocean brightening still lowers AMOC (Xie 2022).</t>
+        </is>
+      </c>
+      <c r="E31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pa510467; pa510522</t>
+        </is>
+      </c>
+      <c r="F31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No dollar value found, so no number is proposed for the workbook.</t>
+        </is>
+      </c>
+      <c r="G31" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no-source</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flag legend</t>
+        </is>
+      </c>
+      <c r="B32" s="401"/>
+      <c r="C32" s="401"/>
+      <c r="D32" s="401"/>
+      <c r="E32" s="401"/>
+      <c r="F32" s="401"/>
+      <c r="G32" s="401"/>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stub = source paper/report has no full text in precis; perplexity-only = only source is a Perplexity ref; hand-FX = currency conversion done by hand with the ECB rate (date and rate recorded); unverified = quote not found in source text; no-source = cell left empty; verified = value and quote read in text held in precis (or arithmetic on such values). Workbook cell values were read from the file with a data-only loader.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A33:G33"/>
+  </mergeCells>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="40" style="167" customWidth="1"/>
@@ -15932,7 +19129,9 @@
     <col min="3" max="3" width="14" style="167" customWidth="1"/>
     <col min="4" max="4" width="68" style="167" customWidth="1"/>
     <col min="5" max="5" width="55" style="167" customWidth="1"/>
-    <col min="6" max="16384" width="8.6640625" style="167"/>
+    <col min="6" max="9" width="8.6640625" style="167"/>
+    <col min="10" max="10" width="120" style="167" customWidth="1"/>
+    <col min="11" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -15969,7 +19168,7 @@
       <c r="E6" s="168"/>
       <c r="F6" s="168"/>
     </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="181" t="s">
         <v>13</v>
       </c>
@@ -15986,8 +19185,13 @@
         <v>17</v>
       </c>
       <c r="F7" s="168"/>
-    </row>
-    <row r="8" spans="1:7" ht="117" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J7" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="117" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="183" t="s">
         <v>18</v>
       </c>
@@ -16004,8 +19208,13 @@
         <v>788</v>
       </c>
       <c r="F8" s="168"/>
-    </row>
-    <row r="9" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J8" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: 1.73e12 particles/s for the best nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="183" t="s">
         <v>21</v>
       </c>
@@ -16020,8 +19229,13 @@
         <v>788</v>
       </c>
       <c r="F9" s="168"/>
-    </row>
-    <row r="10" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="J9" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: 71% of particles fall in 30-1000 nm (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="183" t="s">
         <v>23</v>
       </c>
@@ -16038,6 +19252,11 @@
         <v>789</v>
       </c>
       <c r="F10" s="168"/>
+      <c r="J10" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFLICT: lit count median dry diameter 49.5 nm, GSD 2.01, ~94% of particles below 200 nm for the best nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D); ESMs emit median modal radii of 28.1-72.5 nm (Hirasawa preprint, https://doi.org/10.5194/egusphere-2026-5460). Workbook uses 150 nm.</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="41.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="183" t="s">
@@ -16126,7 +19345,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="183" t="s">
         <v>34</v>
       </c>
@@ -16152,6 +19371,11 @@
       </c>
       <c r="I17" s="185" t="s">
         <v>884</v>
+      </c>
+      <c r="J17" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: 417.4 kW for 814 nozzles = 513 W per nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D); ARIEL prototype 100 nozzles ~55 kW (~550 W each). Workbook 512 W matches.</t>
+        </is>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
@@ -16240,7 +19464,7 @@
       <c r="E22" s="168"/>
       <c r="F22" s="168"/>
     </row>
-    <row r="23" spans="1:9" ht="79" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" ht="79" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="183" t="s">
         <v>40</v>
       </c>
@@ -16257,6 +19481,11 @@
         <v>791</v>
       </c>
       <c r="F23" s="168"/>
+      <c r="J23" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: 0.41 mL/s seawater + 0.3 L/s air per nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
+        </is>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="26" x14ac:dyDescent="0.15">
       <c r="A24" s="183" t="s">
@@ -16292,7 +19521,7 @@
       <c r="E25" s="168"/>
       <c r="F25" s="168"/>
     </row>
-    <row r="26" spans="1:9" ht="39" x14ac:dyDescent="0.15">
+    <row r="26" ht="39" x14ac:dyDescent="0.15">
       <c r="A26" s="183" t="s">
         <v>888</v>
       </c>
@@ -16307,6 +19536,11 @@
       </c>
       <c r="E26" s="168"/>
       <c r="F26" s="168"/>
+      <c r="J26" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found (Harrison 2025 prices only the 15 MPa pressurisation pump, 6.7 kW for 814 nozzles).</t>
+        </is>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="170" t="s">
@@ -16482,9 +19716,359 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="70" customWidth="1"/>
+    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Papers behind the literature notes, and the cells each supports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper</t>
+        </is>
+      </c>
+      <c r="B3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DOI</t>
+        </is>
+      </c>
+      <c r="C3" s="399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cells it supports</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison 2025, Environ. Sci.: Atmos., effervescent nozzle</t>
+        </is>
+      </c>
+      <c r="B4" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
+        </is>
+      </c>
+      <c r="C4" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Technology Description!J8, J9, J10, J17, J23; 2. Cost Inputs!J13, J14; 5a!J12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2026 (preprint), range of MCB radiative forcing across ESMs</t>
+        </is>
+      </c>
+      <c r="B5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
+        </is>
+      </c>
+      <c r="C5" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Technology Description!J10; 6a!N10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate, forcing susceptibility (not checked)</t>
+        </is>
+      </c>
+      <c r="B6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
+        </is>
+      </c>
+      <c r="C6" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!E7:E13 (source of the K per Tg/yr values); 6a!N10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hernandez-Jaramillo, Kelaher &amp; Harrison 2025, plume dispersion review</t>
+        </is>
+      </c>
+      <c r="B7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.3389/fmars.2025.1450175</t>
+        </is>
+      </c>
+      <c r="C7" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5a!J5; 6a!N32</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hernandez-Jaramillo et al. 2025, ERL, first outdoor MCB trial</t>
+        </is>
+      </c>
+      <c r="B8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1088/1748-9326/adccd7</t>
+        </is>
+      </c>
+      <c r="C8" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5a!J12</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stjern et al. 2018, ACP, G4cdnc multi-model ensemble</t>
+        </is>
+      </c>
+      <c r="B9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
+        </is>
+      </c>
+      <c r="C9" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!N16</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Latham et al. 2012, Phil. Trans. R. Soc. A, Marine cloud brightening</t>
+        </is>
+      </c>
+      <c r="B10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
+        </is>
+      </c>
+      <c r="C10" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey tab, section B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hirasawa et al. 2023, GRL, regional MCB and tipping elements</t>
+        </is>
+      </c>
+      <c r="B11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
+        </is>
+      </c>
+      <c r="C11" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b!J19; 6c!J28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xie et al. 2022, ACP, solar geoengineering and the AMOC</t>
+        </is>
+      </c>
+      <c r="B12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-22-4581-2022</t>
+        </is>
+      </c>
+      <c r="C12" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b!J19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tilmes et al. 2014, GRL, regional Arctic climate engineering</t>
+        </is>
+      </c>
+      <c r="B13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1002/2013GL058731</t>
+        </is>
+      </c>
+      <c r="C13" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey tab, section C</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">van Westen, Kliphuis &amp; Dijkstra 2024, Sci. Adv., AMOC early warning</t>
+        </is>
+      </c>
+      <c r="B14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1126/sciadv.adk1189</t>
+        </is>
+      </c>
+      <c r="C14" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey tab, section C</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Burke, Hsiang &amp; Miguel 2015, Nature, temperature and economic production</t>
+        </is>
+      </c>
+      <c r="B15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
+        </is>
+      </c>
+      <c r="C15" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!N44</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kotz, Levermann &amp; Wenz 2024, Nature (not checked)</t>
+        </is>
+      </c>
+      <c r="B16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://doi.org/10.1038/s41586-024-07219-0</t>
+        </is>
+      </c>
+      <c r="C16" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!N45</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nordhaus 2017, NBER w22933, DICE-2016R</t>
+        </is>
+      </c>
+      <c r="B17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no DOI checked</t>
+        </is>
+      </c>
+      <c r="C17" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!N43</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bilal &amp; Kanzig 2024, NBER w32450</t>
+        </is>
+      </c>
+      <c r="B18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no DOI checked</t>
+        </is>
+      </c>
+      <c r="C18" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6a!N45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RRAP CS-06 and CS-07 final reports 2025; RRAP T14 (Harrison et al. 2019)</t>
+        </is>
+      </c>
+      <c r="B19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no DOI</t>
+        </is>
+      </c>
+      <c r="C19" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Cost Inputs!J40; 5a!J25</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PERILS AG industry loss announcements, SCS Cerry (20 Oct 2026) and Raphaela (19 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.perils.org/news</t>
+        </is>
+      </c>
+      <c r="C20" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6b!J19; 6c!J28; Summary tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gallagher Re Q3 2026 Natural Catastrophe and Climate Report, via Reinsurance News (21 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
+        </is>
+      </c>
+      <c r="C21" s="397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Survey tab, section F; Summary tab</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -16493,6 +20077,7 @@
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="69.5" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="10" max="10" width="120" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -16520,7 +20105,7 @@
       <c r="D3" s="357"/>
       <c r="E3" s="357"/>
     </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8"/>
       <c r="B4" s="8" t="s">
         <v>14</v>
@@ -16535,8 +20120,13 @@
       <c r="F4" s="8" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J4" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>63</v>
       </c>
@@ -16553,8 +20143,13 @@
       <c r="F5" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J5" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>67</v>
       </c>
@@ -16571,8 +20166,13 @@
       <c r="F6" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J6" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>71</v>
       </c>
@@ -16587,8 +20187,13 @@
       <c r="F7" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J7" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>891</v>
       </c>
@@ -16603,6 +20208,11 @@
       </c>
       <c r="F8" s="2" t="s">
         <v>894</v>
+      </c>
+      <c r="J8" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16662,7 +20272,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>78</v>
       </c>
@@ -16679,8 +20289,13 @@
       </c>
       <c r="F13" s="354"/>
       <c r="G13" s="354"/>
-    </row>
-    <row r="14" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J13" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: Harrison 2025 (https://doi.org/10.1039/D5EA00073D) needs 814 nozzles for 1e15 CCN/s; workbook 8,141 nozzles is exactly 10x, consistent with its 1e16/s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>80</v>
       </c>
@@ -16696,6 +20311,11 @@
       </c>
       <c r="F14" t="s">
         <v>899</v>
+      </c>
+      <c r="J14" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: Harrison 2025 (https://doi.org/10.1039/D5EA00073D) gives 417.4 kW for 814 nozzles; workbook 4,168 kW is 10x, consistent.</t>
+        </is>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16824,7 +20444,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>95</v>
       </c>
@@ -16842,6 +20462,11 @@
       </c>
       <c r="F25" s="2" t="s">
         <v>752</v>
+      </c>
+      <c r="J25" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No peer-reviewed value found; vessel spec sheets only.</t>
+        </is>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -16918,7 +20543,7 @@
       </c>
       <c r="E30" s="27"/>
     </row>
-    <row r="31" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
         <v>105</v>
       </c>
@@ -16936,6 +20561,11 @@
       </c>
       <c r="F31" s="2" t="s">
         <v>107</v>
+      </c>
+      <c r="J31" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -16965,7 +20595,7 @@
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
     </row>
-    <row r="35" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
         <v>109</v>
       </c>
@@ -16981,6 +20611,11 @@
       </c>
       <c r="F35" s="2" t="s">
         <v>112</v>
+      </c>
+      <c r="J35" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -17029,7 +20664,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
         <v>115</v>
       </c>
@@ -17059,8 +20694,13 @@
       <c r="I40" s="10" t="s">
         <v>903</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J40" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: no published price for this nozzle. RRAP CS-07 final report 2025 gives MeeFog US$50/nozzle (report has no DOI). Workbook range $10-$1,000, selected $100 (H40 = 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
         <v>116</v>
       </c>
@@ -17089,8 +20729,13 @@
       <c r="I41" s="10" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" ht="79" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J41" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found (used-equipment listing only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="79" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>118</v>
       </c>
@@ -17118,8 +20763,13 @@
       <c r="I42" s="10" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J42" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; ballast-water systems are the only comparator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
         <v>120</v>
       </c>
@@ -17145,8 +20795,13 @@
       <c r="I43" s="10" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J43" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found (workbook states nothing published exists).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
         <v>122</v>
       </c>
@@ -17167,6 +20822,11 @@
       </c>
       <c r="G44" s="9" t="s">
         <v>907</v>
+      </c>
+      <c r="J44" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No peer-reviewed value found (trade-press newbuild price basis).</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -17211,7 +20871,7 @@
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
     </row>
-    <row r="49" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -17224,8 +20884,13 @@
       <c r="F49" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J49" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
         <v>130</v>
       </c>
@@ -17238,8 +20903,13 @@
       <c r="F50" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J50" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
         <v>131</v>
       </c>
@@ -17257,8 +20927,13 @@
       <c r="F51" s="33" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J51" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>134</v>
       </c>
@@ -17270,6 +20945,11 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
         <v>135</v>
+      </c>
+      <c r="J52" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
       </c>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -17303,7 +20983,7 @@
       </c>
       <c r="F55" s="8"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>908</v>
       </c>
@@ -17318,6 +20998,11 @@
       </c>
       <c r="E56" t="s">
         <v>832</v>
+      </c>
+      <c r="J56" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No literature value found; assumption.</t>
+        </is>
       </c>
     </row>
     <row r="57" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -23283,14 +26968,16 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="38" style="167" customWidth="1"/>
     <col min="2" max="3" width="18" style="167" customWidth="1"/>
     <col min="4" max="4" width="20" style="167" customWidth="1"/>
     <col min="5" max="5" width="50" style="167" customWidth="1"/>
-    <col min="6" max="16384" width="8.6640625" style="167"/>
+    <col min="6" max="6" width="8.6640625" style="167"/>
+    <col min="7" max="7" width="120" style="167" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -23316,7 +27003,7 @@
       <c r="D4" s="366"/>
       <c r="E4" s="366"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="5" x14ac:dyDescent="0.15">
       <c r="A5" s="235" t="s">
         <v>764</v>
       </c>
@@ -23331,6 +27018,11 @@
       </c>
       <c r="E5" s="235" t="s">
         <v>766</v>
+      </c>
+      <c r="G5" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFLICT: no '~$10B/yr' figure exists anywhere in this workbook (all tabs checked). Cost here is $21.4M/yr per dedicated vessel, $9.3M/yr per piggyback ship and $175B-$18T/yr for 1 K of global cooling (tabs 6b/6c). The ~$10B/yr figure in circulation traces only to a secondary summary of one review; no primary source found.</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -23424,7 +27116,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -23435,7 +27127,7 @@
     <col min="7" max="7" width="39.33203125" customWidth="1"/>
     <col min="8" max="8" width="55" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="10" max="10" width="120" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -23460,7 +27152,7 @@
       <c r="F2" s="368"/>
       <c r="G2" s="368"/>
     </row>
-    <row r="4" spans="1:8" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>57</v>
       </c>
@@ -23473,8 +27165,13 @@
       <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J4" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>371</v>
       </c>
@@ -23492,6 +27189,11 @@
       <c r="G5" s="354"/>
       <c r="H5" s="2" t="s">
         <v>792</v>
+      </c>
+      <c r="J5" s="403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFLICT: no measured value; the plume review lists survival to cloud base as an open research gap (Hernandez-Jaramillo 2025, https://doi.org/10.3389/fmars.2025.1450175). The workbook 0.3 (range 0.1-0.5) has no literature backing.</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:8" ht="79" customHeight="1" x14ac:dyDescent="0.2">
@@ -23599,7 +27301,7 @@
       <c r="F11" s="354"/>
       <c r="G11" s="354"/>
     </row>
-    <row r="12" spans="1:8" ht="41.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" ht="41.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>387</v>
       </c>
@@ -23617,6 +27319,11 @@
       <c r="G12" s="354"/>
       <c r="H12" s="2" t="s">
         <v>795</v>
+      </c>
+      <c r="J12" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lit: ~50 nm activates at 0.5% SS over the GBR (https://doi.org/10.1088/1748-9326/adccd7). CONFLICT: the nozzle's median dry size is 49.5 nm (Harrison 2025, https://doi.org/10.1039/D5EA00073D), so about half its particles sit at or below this threshold, while tab 1 uses 150 nm.</t>
+        </is>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.2">
@@ -23824,7 +27531,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>411</v>
       </c>
@@ -23842,6 +27549,11 @@
       <c r="G25" s="354"/>
       <c r="H25" s="2" t="s">
         <v>797</v>
+      </c>
+      <c r="J25" s="402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source report (RRAP T14, Harrison et al. 2019) has no DOI; value not checked.</t>
+        </is>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
docs(workbook): replace source ids with DOI links; add Nordhaus and Bilal-Kanzig DOIs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118o5nFrXyN5L8uonKyjVV1
</commit_message>
<xml_diff>
--- a/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
+++ b/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
@@ -13833,7 +13833,7 @@
       <c r="I43" s="168"/>
       <c r="N43" s="402" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lit: Nordhaus DICE-2016R (NBER w22933, no DOI checked); not checked against the paper.</t>
+          <t xml:space="preserve">Lit: Nordhaus DICE-2016R, NBER w22933 (https://doi.org/10.3386/w22933); not checked against the paper.</t>
         </is>
       </c>
     </row>
@@ -13881,7 +13881,7 @@
       <c r="I45" s="168"/>
       <c r="N45" s="402" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lit: Bilal &amp; Kanzig 2024 (NBER w32450) coefficient not verified. Kotz et al. 2024 (https://doi.org/10.1038/s41586-024-07219-0): 19% lower world income by 2050 (11-29%), a level not a per-degC rate; not checked.</t>
+          <t xml:space="preserve">Lit: Bilal &amp; Kanzig 2024 (https://doi.org/10.3386/w32450) coefficient not verified. Kotz et al. 2024 (https://doi.org/10.1038/s41586-024-07219-0): 19% lower world income by 2050 (11-29%), a level not a per-degC rate; not checked.</t>
         </is>
       </c>
     </row>
@@ -16064,7 +16064,7 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="400" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Survey of the state of the art on this workbook's inputs and outputs. Flags: stub, perplexity-only, hand-FX, unverified, no-source, verified (legend on the Summary tab). Empty value cells mean no source was found. Source handles are the precis knowledge-graph ids.</t>
+          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Survey of the state of the art on this workbook's inputs and outputs. Flags: stub, perplexity-only, hand-FX, unverified, no-source, verified (legend on the Summary tab). Empty value cells mean no source was found. Source links are DOIs or URLs.</t>
         </is>
       </c>
     </row>
@@ -16091,7 +16091,7 @@
       </c>
       <c r="E3" s="399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Source handle</t>
+          <t xml:space="preserve">Source link</t>
         </is>
       </c>
       <c r="F3" s="399" t="inlineStr">
@@ -16145,7 +16145,7 @@
       </c>
       <c r="E5" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238582</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F5" s="397" t="inlineStr">
@@ -16185,7 +16185,7 @@
       </c>
       <c r="E6" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238582</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F6" s="397" t="inlineStr">
@@ -16221,7 +16221,7 @@
       <c r="D7" s="397"/>
       <c r="E7" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238583</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F7" s="397" t="inlineStr">
@@ -16261,7 +16261,7 @@
       </c>
       <c r="E8" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238583</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F8" s="397" t="inlineStr">
@@ -16301,7 +16301,7 @@
       </c>
       <c r="E9" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238583</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F9" s="397" t="inlineStr">
@@ -16341,7 +16341,7 @@
       </c>
       <c r="E10" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238584</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F10" s="397" t="inlineStr">
@@ -16381,7 +16381,7 @@
       </c>
       <c r="E11" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238581</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F11" s="397" t="inlineStr">
@@ -16421,7 +16421,7 @@
       </c>
       <c r="E12" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513654 (RRAP CS-07 final report 2025, pp.31,35 per workbook); web:513652 (CS-06)</t>
+          <t xml:space="preserve">https://gbrrestoration.org/wp-content/uploads/2026/06/RRAP-CS-07_FINAL-REPORT-2025.pdf  https://gbrrestoration.org/wp-content/uploads/2026/06/RRAP-CS-06_FINAL-REPORT-2025.pdf</t>
         </is>
       </c>
       <c r="F12" s="397" t="inlineStr">
@@ -16573,7 +16573,7 @@
       </c>
       <c r="E17" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509685 / pc5154182</t>
+          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
         </is>
       </c>
       <c r="F17" s="397" t="inlineStr">
@@ -16609,7 +16609,7 @@
       <c r="D18" s="397"/>
       <c r="E18" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509685 / pc5154182</t>
+          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
         </is>
       </c>
       <c r="F18" s="397" t="inlineStr">
@@ -16649,7 +16649,7 @@
       </c>
       <c r="E19" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509690 / pc5153550</t>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
         </is>
       </c>
       <c r="F19" s="397" t="inlineStr">
@@ -16689,7 +16689,7 @@
       </c>
       <c r="E20" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509690 / pc5153551</t>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
         </is>
       </c>
       <c r="F20" s="397" t="inlineStr">
@@ -16729,7 +16729,7 @@
       </c>
       <c r="E21" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513649 / pc5238641</t>
+          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
         </is>
       </c>
       <c r="F21" s="397" t="inlineStr">
@@ -16769,7 +16769,7 @@
       </c>
       <c r="E22" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513649 / pc5238641</t>
+          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
         </is>
       </c>
       <c r="F22" s="397" t="inlineStr">
@@ -16807,7 +16807,7 @@
       <c r="D23" s="397"/>
       <c r="E23" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513649 / pc5238641</t>
+          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
         </is>
       </c>
       <c r="F23" s="397" t="inlineStr">
@@ -16847,7 +16847,7 @@
       </c>
       <c r="E24" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513648</t>
+          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
         </is>
       </c>
       <c r="F24" s="397" t="inlineStr">
@@ -16887,7 +16887,7 @@
       </c>
       <c r="E25" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513648</t>
+          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
         </is>
       </c>
       <c r="F25" s="397" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="E26" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513648</t>
+          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
         </is>
       </c>
       <c r="F26" s="397" t="inlineStr">
@@ -16965,7 +16965,7 @@
       </c>
       <c r="E27" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510540 / pc5168648</t>
+          <t xml:space="preserve">https://doi.org/10.3389/fmars.2025.1450175</t>
         </is>
       </c>
       <c r="F27" s="397" t="inlineStr">
@@ -17005,7 +17005,7 @@
       </c>
       <c r="E28" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513655 (RRAP T14, Harrison et al. 2019)</t>
+          <t xml:space="preserve">https://gbrrestoration.org/wp-content/uploads/2020/09/T14-Environmental-Modelling-of-Large-Scale-SRM_v3.03-3.pdf</t>
         </is>
       </c>
       <c r="F28" s="397" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="E30" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509690 / pc5153551</t>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
         </is>
       </c>
       <c r="F30" s="397" t="inlineStr">
@@ -17095,7 +17095,7 @@
       <c r="D31" s="397"/>
       <c r="E31" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa509690 / pc5153551</t>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
         </is>
       </c>
       <c r="F31" s="397" t="inlineStr">
@@ -17133,7 +17133,7 @@
       <c r="D32" s="397"/>
       <c r="E32" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510467 / pc5166683</t>
+          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
         </is>
       </c>
       <c r="F32" s="397" t="inlineStr">
@@ -17171,7 +17171,7 @@
       <c r="D33" s="397"/>
       <c r="E33" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510467 / pc5166639</t>
+          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
         </is>
       </c>
       <c r="F33" s="397" t="inlineStr">
@@ -17209,7 +17209,7 @@
       <c r="D34" s="397"/>
       <c r="E34" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510522 / pc5179359</t>
+          <t xml:space="preserve">https://doi.org/10.5194/acp-22-4581-2022</t>
         </is>
       </c>
       <c r="F34" s="397" t="inlineStr">
@@ -17247,7 +17247,7 @@
       <c r="D35" s="397"/>
       <c r="E35" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510511 / pc5180602</t>
+          <t xml:space="preserve">https://doi.org/10.1002/2013GL058731</t>
         </is>
       </c>
       <c r="F35" s="397" t="inlineStr">
@@ -17287,7 +17287,7 @@
       </c>
       <c r="E36" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510518 / pc5179664</t>
+          <t xml:space="preserve">https://doi.org/10.1126/sciadv.adk1189</t>
         </is>
       </c>
       <c r="F36" s="397" t="inlineStr">
@@ -17315,11 +17315,7 @@
       <c r="B37" s="397"/>
       <c r="C37" s="397"/>
       <c r="D37" s="397"/>
-      <c r="E37" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">td510496 (no linked papers)</t>
-        </is>
-      </c>
+      <c r="E37" s="397"/>
       <c r="F37" s="397"/>
       <c r="G37" s="397" t="inlineStr">
         <is>
@@ -17341,11 +17337,7 @@
       <c r="B38" s="397"/>
       <c r="C38" s="397"/>
       <c r="D38" s="397"/>
-      <c r="E38" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">td510496 (no linked papers)</t>
-        </is>
-      </c>
+      <c r="E38" s="397"/>
       <c r="F38" s="397"/>
       <c r="G38" s="397" t="inlineStr">
         <is>
@@ -17371,11 +17363,7 @@
         </is>
       </c>
       <c r="D39" s="397"/>
-      <c r="E39" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">td510498</t>
-        </is>
-      </c>
+      <c r="E39" s="397"/>
       <c r="F39" s="397"/>
       <c r="G39" s="397" t="inlineStr">
         <is>
@@ -17423,7 +17411,7 @@
       </c>
       <c r="E41" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">perplexity-reasoning:510558 [42] PMC6784395</t>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6784395/</t>
         </is>
       </c>
       <c r="F41" s="397" t="inlineStr">
@@ -17463,11 +17451,7 @@
           <t xml:space="preserve">Perplexity annualises to ~$26B per W/m2-yr</t>
         </is>
       </c>
-      <c r="E42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-reasoning:510558 [33]</t>
-        </is>
-      </c>
+      <c r="E42" s="397"/>
       <c r="F42" s="397" t="inlineStr">
         <is>
           <t xml:space="preserve">Perplexity answer; underlying NASEM text not read</t>
@@ -17505,11 +17489,7 @@
           <t xml:space="preserve">media/interview estimate</t>
         </is>
       </c>
-      <c r="E43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-reasoning:510558 [33]</t>
-        </is>
-      </c>
+      <c r="E43" s="397"/>
       <c r="F43" s="397" t="inlineStr">
         <is>
           <t xml:space="preserve">Perplexity answer; underlying source not read</t>
@@ -17547,7 +17527,7 @@
       </c>
       <c r="E44" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">perplexity-reasoning:510558 [44]</t>
+          <t xml:space="preserve">https://doi.org/10.1088/2515-7620/ad2f71</t>
         </is>
       </c>
       <c r="F44" s="397" t="inlineStr">
@@ -17597,12 +17577,12 @@
       <c r="D46" s="397"/>
       <c r="E46" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">(no paper in precis)</t>
+          <t xml:space="preserve">https://doi.org/10.3386/w22933</t>
         </is>
       </c>
       <c r="F46" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nordhaus (2017), NBER w22933, as cited in workbook tab 6a G43</t>
+          <t xml:space="preserve">Nordhaus (2016), NBER w22933 (DICE-2016R), as cited in workbook tab 6a G43</t>
         </is>
       </c>
       <c r="G46" s="397" t="inlineStr">
@@ -17637,7 +17617,7 @@
       </c>
       <c r="E47" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510562</t>
+          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
         </is>
       </c>
       <c r="F47" s="397" t="inlineStr">
@@ -17673,7 +17653,7 @@
       <c r="D48" s="397"/>
       <c r="E48" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">perplexity-reasoning:510558</t>
+          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
         </is>
       </c>
       <c r="F48" s="397" t="inlineStr">
@@ -17709,7 +17689,7 @@
       <c r="D49" s="397"/>
       <c r="E49" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">(no paper in precis)</t>
+          <t xml:space="preserve">https://doi.org/10.3386/w32450</t>
         </is>
       </c>
       <c r="F49" s="397" t="inlineStr">
@@ -17749,7 +17729,7 @@
       </c>
       <c r="E50" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">perplexity-reasoning:510558</t>
+          <t xml:space="preserve">https://doi.org/10.1038/s41586-024-07219-0</t>
         </is>
       </c>
       <c r="F50" s="397" t="inlineStr">
@@ -17781,11 +17761,7 @@
         </is>
       </c>
       <c r="D51" s="397"/>
-      <c r="E51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-reasoning:510558</t>
-        </is>
-      </c>
+      <c r="E51" s="397"/>
       <c r="F51" s="397" t="inlineStr">
         <is>
           <t xml:space="preserve">Perplexity answer</t>
@@ -17837,7 +17813,7 @@
       </c>
       <c r="E53" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026</t>
         </is>
       </c>
       <c r="F53" s="397" t="inlineStr">
@@ -17877,7 +17853,7 @@
       </c>
       <c r="E54" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513650</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
         </is>
       </c>
       <c r="F54" s="397" t="inlineStr">
@@ -17913,7 +17889,7 @@
       <c r="D55" s="397"/>
       <c r="E55" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651 + web:513650</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
         </is>
       </c>
       <c r="F55" s="397" t="inlineStr">
@@ -17949,7 +17925,7 @@
       <c r="D56" s="397"/>
       <c r="E56" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651 + web:513650</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
         </is>
       </c>
       <c r="F56" s="397" t="inlineStr">
@@ -17985,7 +17961,7 @@
       <c r="D57" s="397"/>
       <c r="E57" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651 + api.frankfurter.app</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://api.frankfurter.app</t>
         </is>
       </c>
       <c r="F57" s="397" t="inlineStr">
@@ -18021,7 +17997,7 @@
       <c r="D58" s="397"/>
       <c r="E58" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513650 + api.frankfurter.app</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
         </is>
       </c>
       <c r="F58" s="397" t="inlineStr">
@@ -18061,7 +18037,7 @@
       </c>
       <c r="E59" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651 + web:513650 + api.frankfurter.app</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
         </is>
       </c>
       <c r="F59" s="397" t="inlineStr">
@@ -18101,12 +18077,12 @@
       </c>
       <c r="E60" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513656</t>
+          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
         </is>
       </c>
       <c r="F60" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinsurance News, 21 Oct 2026, reporting Gallagher Re Q3 2026 Natural Catastrophe and Climate Report (primary report page web:513653 has no extractable text)</t>
+          <t xml:space="preserve">Reinsurance News, 21 Oct 2026, reporting Gallagher Re Q3 2026 Natural Catastrophe and Climate Report (the primary Gallagher Re report page has no extractable text)</t>
         </is>
       </c>
       <c r="G60" s="397" t="inlineStr">
@@ -18141,7 +18117,7 @@
       </c>
       <c r="E61" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513656 vs web:513650</t>
+          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
         </is>
       </c>
       <c r="F61" s="397" t="inlineStr">
@@ -18181,7 +18157,7 @@
       </c>
       <c r="E62" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513656</t>
+          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
         </is>
       </c>
       <c r="F62" s="397" t="inlineStr">
@@ -18260,7 +18236,7 @@
       </c>
       <c r="E3" s="399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Survey handle</t>
+          <t xml:space="preserve">Source link</t>
         </is>
       </c>
       <c r="F3" s="399" t="inlineStr">
@@ -18317,7 +18293,7 @@
       </c>
       <c r="E6" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">perplexity-reasoning:510558 [42]</t>
+          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6784395/</t>
         </is>
       </c>
       <c r="F6" s="397" t="inlineStr">
@@ -18365,7 +18341,7 @@
       </c>
       <c r="E8" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238582, pc5238583</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
         </is>
       </c>
       <c r="F8" s="397" t="inlineStr">
@@ -18493,7 +18469,7 @@
       </c>
       <c r="E12" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513647 / pc5238581; pa513649 / pc5238641</t>
+          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D  https://doi.org/10.5194/egusphere-2026-5460</t>
         </is>
       </c>
       <c r="F12" s="397" t="inlineStr">
@@ -18530,7 +18506,7 @@
       </c>
       <c r="E13" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa513649 / pc5238641; pa509690 / pc5153550</t>
+          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460  https://doi.org/10.5194/acp-18-621-2018</t>
         </is>
       </c>
       <c r="F13" s="397" t="inlineStr">
@@ -18600,7 +18576,7 @@
       </c>
       <c r="E15" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510562; perplexity-reasoning:510558</t>
+          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
         </is>
       </c>
       <c r="F15" s="397" t="inlineStr">
@@ -18780,7 +18756,7 @@
       </c>
       <c r="E21" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651, web:513650, api.frankfurter.app</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
         </is>
       </c>
       <c r="F21" s="397" t="inlineStr">
@@ -18976,7 +18952,7 @@
       </c>
       <c r="E27" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513656</t>
+          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
         </is>
       </c>
       <c r="F27" s="397" t="inlineStr">
@@ -19033,7 +19009,7 @@
       </c>
       <c r="E30" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">web:513651, web:513650</t>
+          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
         </is>
       </c>
       <c r="F30" s="397" t="inlineStr">
@@ -19070,7 +19046,7 @@
       </c>
       <c r="E31" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">pa510467; pa510522</t>
+          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314  https://doi.org/10.5194/acp-22-4581-2022</t>
         </is>
       </c>
       <c r="F31" s="397" t="inlineStr">
@@ -19977,12 +19953,12 @@
     <row r="17">
       <c r="A17" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nordhaus 2017, NBER w22933, DICE-2016R</t>
+          <t xml:space="preserve">Nordhaus 2016, NBER w22933, DICE-2016R (Projections and Uncertainties About Climate Change in an Era of Minimal Climate Policies)</t>
         </is>
       </c>
       <c r="B17" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">no DOI checked</t>
+          <t xml:space="preserve">https://doi.org/10.3386/w22933</t>
         </is>
       </c>
       <c r="C17" s="397" t="inlineStr">
@@ -19994,12 +19970,12 @@
     <row r="18">
       <c r="A18" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bilal &amp; Kanzig 2024, NBER w32450</t>
+          <t xml:space="preserve">Bilal &amp; Kanzig 2024, NBER w32450, The Macroeconomic Impact of Climate Change: Global vs. Local Temperature</t>
         </is>
       </c>
       <c r="B18" s="397" t="inlineStr">
         <is>
-          <t xml:space="preserve">no DOI checked</t>
+          <t xml:space="preserve">https://doi.org/10.3386/w32450</t>
         </is>
       </c>
       <c r="C18" s="397" t="inlineStr">

</xml_diff>

<commit_message>
feat(colab): uncertainty dashboard; restore Tito's workbook, annotations move to CSVs
Tornado, Monte Carlo (0.9 ms/run), sweeps, literature models beside Tito's
formulas; ranges/survey/summary/sources/literature_models CSVs; runtime
annotated-xlsx export.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118o5nFrXyN5L8uonKyjVV1
</commit_message>
<xml_diff>
--- a/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
+++ b/Draft MCB TEA and Cost Benefit TJ 10122026.xlsx
@@ -25,9 +25,6 @@
     <sheet name="6b. Benefit - Global - Vessel" sheetId="14" r:id="rId15"/>
     <sheet name="6c. Benefit - Global Piggyback" sheetId="15" r:id="rId16"/>
     <sheet name="References" sheetId="17" r:id="rId17"/>
-    <sheet name="Survey (added by precis)" sheetId="19" r:id="rId101"/>
-    <sheet name="Summary (added by precis)" sheetId="20" r:id="rId102"/>
-    <sheet name="Sources (added by precis)" sheetId="21" r:id="rId103"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -3020,7 +3017,7 @@
     <numFmt numFmtId="180" formatCode="\$#,##0.0"/>
     <numFmt numFmtId="181" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="62" x14ac:knownFonts="1">
+  <fonts count="57" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3408,36 +3405,8 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF375623"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3501,24 +3470,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF8EFA00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFD966"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3668,7 +3619,7 @@
     <xf numFmtId="44" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="56" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="404">
+  <cellXfs count="397">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4605,27 +4556,6 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -13019,7 +12949,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:N82"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="40" style="167" customWidth="1"/>
@@ -13032,9 +12962,7 @@
     <col min="8" max="8" width="17.83203125" style="167" customWidth="1"/>
     <col min="9" max="9" width="20" style="167" customWidth="1"/>
     <col min="10" max="10" width="33.5" style="167" customWidth="1"/>
-    <col min="11" max="13" width="8.6640625" style="167"/>
-    <col min="14" max="14" width="120" style="167" customWidth="1"/>
-    <col min="15" max="16384" width="8.6640625" style="167"/>
+    <col min="11" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
@@ -13092,7 +13020,7 @@
       <c r="F5" s="363"/>
       <c r="G5" s="363"/>
     </row>
-    <row r="6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="111" t="s">
         <v>614</v>
       </c>
@@ -13112,11 +13040,6 @@
       <c r="G6" s="111" t="s">
         <v>268</v>
       </c>
-      <c r="N6" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
-        </is>
-      </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="270" t="s">
@@ -13183,7 +13106,7 @@
       </c>
       <c r="H9" s="387"/>
     </row>
-    <row r="10" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="270" t="s">
         <v>626</v>
       </c>
@@ -13204,11 +13127,6 @@
         <v>627</v>
       </c>
       <c r="H10" s="387"/>
-      <c r="N10" s="403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFLICT: these K-per-Tg/yr values come from Hirasawa 2026 (https://doi.org/10.1175/JCLI-D-25-0337.1), not checked (full text unavailable). The preprint (https://doi.org/10.5194/egusphere-2026-5460) finds emissions for -2 W/m2 span 7-93 Tg/yr across nine models (13x); the workbook spread is 31x (0.236 vs 0.00754).</t>
-        </is>
-      </c>
     </row>
     <row r="11" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="270" t="s">
@@ -13294,7 +13212,7 @@
       <c r="F15" s="363"/>
       <c r="G15" s="363"/>
     </row>
-    <row r="16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="274" t="s">
         <v>836</v>
       </c>
@@ -13315,11 +13233,6 @@
         <v>834</v>
       </c>
       <c r="H16" s="387"/>
-      <c r="N16" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: for the same 50% droplet-number increase, 9 ESMs give ERF -0.6 to -2.5 W/m2 (4.2x), median -1.9 (Stjern 2018, https://doi.org/10.5194/acp-18-621-2018).</t>
-        </is>
-      </c>
     </row>
     <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="274" t="s">
@@ -13553,7 +13466,7 @@
       </c>
       <c r="I31" s="390"/>
     </row>
-    <row r="32" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="168" t="s">
         <v>653</v>
       </c>
@@ -13569,11 +13482,6 @@
       <c r="G32" s="201"/>
       <c r="H32" s="339"/>
       <c r="I32" s="339"/>
-      <c r="N32" s="403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFLICT: no literature value for survival to cloud base; open gap (https://doi.org/10.3389/fmars.2025.1450175). See tab 5a B5.</t>
-        </is>
-      </c>
     </row>
     <row r="33" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="111" t="s">
@@ -13813,7 +13721,7 @@
       <c r="H42" s="168"/>
       <c r="I42" s="168"/>
     </row>
-    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="274" t="s">
         <v>951</v>
       </c>
@@ -13831,13 +13739,8 @@
       </c>
       <c r="H43" s="168"/>
       <c r="I43" s="168"/>
-      <c r="N43" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: Nordhaus DICE-2016R, NBER w22933 (https://doi.org/10.3386/w22933); not checked against the paper.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="274" t="s">
         <v>952</v>
       </c>
@@ -13855,13 +13758,8 @@
       </c>
       <c r="H44" s="168"/>
       <c r="I44" s="168"/>
-      <c r="N44" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: Burke et al. 2015 (https://doi.org/10.1038/nature15725) reports a non-linear response, ~23% lower global income by 2100 unmitigated (secondary summary), not a per-degC rate; 3.3%/degC is the workbook's own conversion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="274" t="s">
         <v>953</v>
       </c>
@@ -13879,11 +13777,6 @@
       </c>
       <c r="H45" s="168"/>
       <c r="I45" s="168"/>
-      <c r="N45" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: Bilal &amp; Kanzig 2024 (https://doi.org/10.3386/w32450) coefficient not verified. Kotz et al. 2024 (https://doi.org/10.1038/s41586-024-07219-0): 19% lower world income by 2050 (11-29%), a level not a per-degC rate; not checked.</t>
-        </is>
-      </c>
     </row>
     <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="168"/>
@@ -14280,7 +14173,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="38" style="167" customWidth="1"/>
@@ -14291,9 +14184,7 @@
     <col min="6" max="6" width="25.5" style="167" customWidth="1"/>
     <col min="7" max="7" width="46" style="167" customWidth="1"/>
     <col min="8" max="8" width="10" style="167" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" style="167"/>
-    <col min="10" max="10" width="120" style="167" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="167"/>
+    <col min="9" max="16384" width="8.83203125" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -14516,7 +14407,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="234" t="s">
         <v>667</v>
       </c>
@@ -14531,11 +14422,6 @@
       </c>
       <c r="E19" s="234" t="s">
         <v>415</v>
-      </c>
-      <c r="J19" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scale cross-check: damage per degC already contains storm damage. 2026 EU hail/storm insured losses were EUR 6.1B for two events (PERILS, https://www.perils.org/news), ~0.2% of the central $3,630B per K-year; do not add as a separate line. AMOC effect on this benefit is model-dependent (Hirasawa 2023 https://doi.org/10.1029/2023GL104314; Xie 2022 https://doi.org/10.5194/acp-22-4581-2022).</t>
-        </is>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.15">
@@ -14756,7 +14642,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="42" style="167" customWidth="1"/>
@@ -14767,9 +14653,7 @@
     <col min="6" max="6" width="22" style="167" customWidth="1"/>
     <col min="7" max="7" width="18" style="167" customWidth="1"/>
     <col min="8" max="8" width="10" style="167" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" style="167"/>
-    <col min="10" max="10" width="120" style="167" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="167"/>
+    <col min="9" max="16384" width="8.83203125" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -15149,7 +15033,7 @@
       <c r="G27" s="168"/>
       <c r="H27" s="168"/>
     </row>
-    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="234" t="s">
         <v>667</v>
       </c>
@@ -15167,11 +15051,6 @@
       </c>
       <c r="G28" s="168"/>
       <c r="H28" s="168"/>
-      <c r="J28" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scale cross-check: damage per degC already contains storm damage. 2026 EU hail/storm insured losses were EUR 6.1B for two events (PERILS, https://www.perils.org/news), ~0.2% of the central $3,630B per K-year. See tab 6b note.</t>
-        </is>
-      </c>
     </row>
     <row r="29" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="304" t="s">
@@ -16043,3061 +15922,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-  </sheetPr>
-  <dimension ref="A1:H62"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="70" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="48" customHeight="1">
-      <c r="A1" s="400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Survey of the state of the art on this workbook's inputs and outputs. Flags: stub, perplexity-only, hand-FX, unverified, no-source, verified (legend on the Summary tab). Empty value cells mean no source was found. Source links are DOIs or URLs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quantity</t>
-        </is>
-      </c>
-      <c r="B3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value</t>
-        </is>
-      </c>
-      <c r="C3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unit</t>
-        </is>
-      </c>
-      <c r="D3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Range</t>
-        </is>
-      </c>
-      <c r="E3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source link</t>
-        </is>
-      </c>
-      <c r="F3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Citation</t>
-        </is>
-      </c>
-      <c r="G3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quote / locator</t>
-        </is>
-      </c>
-      <c r="H3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flag</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A. Spray / nozzle cost and rate</t>
-        </is>
-      </c>
-      <c r="B4" s="401"/>
-      <c r="C4" s="401"/>
-      <c r="D4" s="401"/>
-      <c r="E4" s="401"/>
-      <c r="F4" s="401"/>
-      <c r="G4" s="401"/>
-      <c r="H4" s="401"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nozzle particle production rate (best nozzle tested)</t>
-        </is>
-      </c>
-      <c r="B5" s="397">
-        <v>1730000000000.0</v>
-      </c>
-      <c r="C5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">particles/s per nozzle</t>
-        </is>
-      </c>
-      <c r="D5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">71% of particles within 30-1000 nm dry diameter</t>
-        </is>
-      </c>
-      <c r="E5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"This nozzle produces an estimated 1.73×10^12 s -1 droplets from 0.41 mL s -1 filtered seawater (and 0.3 L s -1 of air) with 71% of those particles being within the assumed MCB effectiveness range of 30 to 1000 nm dry diameter."</t>
-        </is>
-      </c>
-      <c r="H5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seawater flow per nozzle</t>
-        </is>
-      </c>
-      <c r="B6" s="397">
-        <v>0.41</v>
-      </c>
-      <c r="C6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mL/s</t>
-        </is>
-      </c>
-      <c r="D6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">air 0.3 L/s</t>
-        </is>
-      </c>
-      <c r="E6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">same sentence as above</t>
-        </is>
-      </c>
-      <c r="H6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nozzles needed for 1e15 CCN/s (30-1000 nm)</t>
-        </is>
-      </c>
-      <c r="B7" s="397">
-        <v>814</v>
-      </c>
-      <c r="C7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nozzles</t>
-        </is>
-      </c>
-      <c r="D7" s="397"/>
-      <c r="E7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"To reach a target CCN production rate of 10^15 s -1 within the 30- 1000nm size range would require 814 of this current effervescent nozzle."</t>
-        </is>
-      </c>
-      <c r="H7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spray-equipment power for 814 nozzles (compressor 410.7 kW + pump 6.7 kW)</t>
-        </is>
-      </c>
-      <c r="B8" s="397">
-        <v>417.4</v>
-      </c>
-      <c r="C8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kW</t>
-        </is>
-      </c>
-      <c r="D8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">compressor eff. 0.72, pump eff. 0.75, 15 MPa</t>
-        </is>
-      </c>
-      <c r="E8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Combined this spraying equipment would require 417.4 kW to supply the 814 nozzles."</t>
-        </is>
-      </c>
-      <c r="H8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Power per nozzle (derived: 417.4 kW / 814)</t>
-        </is>
-      </c>
-      <c r="B9" s="397">
-        <v>0.513</v>
-      </c>
-      <c r="C9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kW per nozzle</t>
-        </is>
-      </c>
-      <c r="D9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook uses 512 W (tab 3a, tornado input C49)</t>
-        </is>
-      </c>
-      <c r="E9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arithmetic on the two quoted figures above; matches the workbook's 512 W.</t>
-        </is>
-      </c>
-      <c r="H9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARIEL prototype: 100 nozzles power</t>
-        </is>
-      </c>
-      <c r="B10" s="397">
-        <v>55</v>
-      </c>
-      <c r="C10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kW (approx.)</t>
-        </is>
-      </c>
-      <c r="D10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">implies ~550 W per nozzle</t>
-        </is>
-      </c>
-      <c r="E10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"a prototype of 100 nozzles requiring approximately 55 kW facilitated the initial outdoor tests"</t>
-        </is>
-      </c>
-      <c r="H10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dry particle size of best nozzle (count median diameter)</t>
-        </is>
-      </c>
-      <c r="B11" s="397">
-        <v>49.5</v>
-      </c>
-      <c r="C11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nm</t>
-        </is>
-      </c>
-      <c r="D11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GSD 2.01; ~94% of particles below 200 nm</t>
-        </is>
-      </c>
-      <c r="E11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison (2025), Environ. Sci.: Atmos., doi:10.1039/D5EA00073D (accepted manuscript)</t>
-        </is>
-      </c>
-      <c r="G11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"had a CMD of 49.5 nm dry particle diameter and a GSD of 2.01". The workbook's design point is 150 nm (tab 6a B20); see Summary.</t>
-        </is>
-      </c>
-      <c r="H11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nozzle + manifold unit price</t>
-        </is>
-      </c>
-      <c r="B12" s="397">
-        <v>50</v>
-      </c>
-      <c r="C12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$/nozzle (MeeFog price as cited by the workbook)</t>
-        </is>
-      </c>
-      <c r="D12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook bracket $10-$1,000; base $100</t>
-        </is>
-      </c>
-      <c r="E12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://gbrrestoration.org/wp-content/uploads/2026/06/RRAP-CS-07_FINAL-REPORT-2025.pdf  https://gbrrestoration.org/wp-content/uploads/2026/06/RRAP-CS-06_FINAL-REPORT-2025.pdf</t>
-        </is>
-      </c>
-      <c r="F12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reef Restoration &amp; Adaptation Program CS-07 / CS-06 final reports 2025</t>
-        </is>
-      </c>
-      <c r="G12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value is the workbook's/strand's citation. PDF is cached but has no extracted text, so the figure could not be read in precis.</t>
-        </is>
-      </c>
-      <c r="H12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Compression + generation capex</t>
-        </is>
-      </c>
-      <c r="B13" s="397"/>
-      <c r="C13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$/kW</t>
-        </is>
-      </c>
-      <c r="D13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook uses 1,500 $/kW</t>
-        </is>
-      </c>
-      <c r="E13" s="397"/>
-      <c r="F13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook cites a used 200 hp CNG compressor yard listing; not in precis</t>
-        </is>
-      </c>
-      <c r="G13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No source in the graph.</t>
-        </is>
-      </c>
-      <c r="H13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vessel purchase price (70-80 m PSV newbuild)</t>
-        </is>
-      </c>
-      <c r="B14" s="397"/>
-      <c r="C14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$</t>
-        </is>
-      </c>
-      <c r="D14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook uses $30M (22.5-56M)</t>
-        </is>
-      </c>
-      <c r="E14" s="397"/>
-      <c r="F14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook cites Clarksons via Riviera Maritime Media; not in precis</t>
-        </is>
-      </c>
-      <c r="G14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No source in the graph.</t>
-        </is>
-      </c>
-      <c r="H14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vessel fuel burn and price (16,000 L/d underway, $0.9/L), crew, charter</t>
-        </is>
-      </c>
-      <c r="B15" s="397"/>
-      <c r="C15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">various</t>
-        </is>
-      </c>
-      <c r="D15" s="397"/>
-      <c r="E15" s="397"/>
-      <c r="F15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook cites PSV spec sheets and assumptions; none in precis</t>
-        </is>
-      </c>
-      <c r="G15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No source in the graph.</t>
-        </is>
-      </c>
-      <c r="H15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">B. Forcing per unit effort and climate-model spread</t>
-        </is>
-      </c>
-      <c r="B16" s="401"/>
-      <c r="C16" s="401"/>
-      <c r="D16" s="401"/>
-      <c r="E16" s="401"/>
-      <c r="F16" s="401"/>
-      <c r="G16" s="401"/>
-      <c r="H16" s="401"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spray vessels to offset CO2 doubling (Flettner design, Salter et al.)</t>
-        </is>
-      </c>
-      <c r="B17" s="397">
-        <v>1500</v>
-      </c>
-      <c r="C17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vessels</t>
-        </is>
-      </c>
-      <c r="D17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">each ~150 kW (wind-derived)</t>
-        </is>
-      </c>
-      <c r="E17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
-        </is>
-      </c>
-      <c r="F17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Latham et al. (2012), 'Marine cloud brightening'</t>
-        </is>
-      </c>
-      <c r="G17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"about 1500 spray vessels, each consuming about 150 kW (derived from the wind), would be required to produce the globally averaged negative forcing of −3.7 W m−2 required to balance carbon dioxide doubling."</t>
-        </is>
-      </c>
-      <c r="H17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Forcing target for those vessels</t>
-        </is>
-      </c>
-      <c r="B18" s="397">
-        <v>-3.7</v>
-      </c>
-      <c r="C18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">W/m2 (global mean)</t>
-        </is>
-      </c>
-      <c r="D18" s="397"/>
-      <c r="E18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
-        </is>
-      </c>
-      <c r="F18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Latham et al. (2012)</t>
-        </is>
-      </c>
-      <c r="G18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">same sentence as above</t>
-        </is>
-      </c>
-      <c r="H18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ensemble effective radiative forcing, +50% CDNC in low marine clouds, 9 ESMs</t>
-        </is>
-      </c>
-      <c r="B19" s="397">
-        <v>-1.9</v>
-      </c>
-      <c r="C19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">W/m2 (median)</t>
-        </is>
-      </c>
-      <c r="D19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-0.6 to -2.5</t>
-        </is>
-      </c>
-      <c r="E19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="F19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
-        </is>
-      </c>
-      <c r="G19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"The model ensemble median effective radiative forcing (ERF) amounts to −1.9 W m−2, with a substantial inter-model spread of −0.6 to −2.5 W m−2."</t>
-        </is>
-      </c>
-      <c r="H19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ensemble global cooling for that forcing (2020-2069 vs RCP4.5)</t>
-        </is>
-      </c>
-      <c r="B20" s="397">
-        <v>-0.96</v>
-      </c>
-      <c r="C20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K (median)</t>
-        </is>
-      </c>
-      <c r="D20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-0.17 to -1.21</t>
-        </is>
-      </c>
-      <c r="E20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="F20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
-        </is>
-      </c>
-      <c r="G20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"a median of (for years 2020–2069) −0.96 [−0.17 to −1.21] K relative to the RCP4.5 scenario"</t>
-        </is>
-      </c>
-      <c r="H20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sea-salt emission needed for -2 W/m2, lowest model</t>
-        </is>
-      </c>
-      <c r="B21" s="397">
-        <v>7</v>
-      </c>
-      <c r="C21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tg/yr</t>
-        </is>
-      </c>
-      <c r="D21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7 to 93 Tg/yr across nine models (13x)</t>
-        </is>
-      </c>
-      <c r="E21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="F21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="G21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"iSSA mass emissions to get −2 Wm−2 ranging from 7 Tg yr−1 to 93 Tg yr−1 in models."</t>
-        </is>
-      </c>
-      <c r="H21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sea-salt emission needed for -2 W/m2, highest model</t>
-        </is>
-      </c>
-      <c r="B22" s="397">
-        <v>93</v>
-      </c>
-      <c r="C22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tg/yr</t>
-        </is>
-      </c>
-      <c r="D22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">see above</t>
-        </is>
-      </c>
-      <c r="E22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="F22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="G22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">same sentence as above</t>
-        </is>
-      </c>
-      <c r="H22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emitted median modal radius across ESMs</t>
-        </is>
-      </c>
-      <c r="B23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28.1 to 72.5</t>
-        </is>
-      </c>
-      <c r="C23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nm</t>
-        </is>
-      </c>
-      <c r="D23" s="397"/>
-      <c r="E23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="F23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. (2026 preprint), 'On the Range of Marine Cloud Brightening Radiative Forcing across Earth System Models', doi:10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="G23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"the ESMs use median modal radii ranging from 28.1nm to 72.5nm, resulting in major differences in CCN concentration."</t>
-        </is>
-      </c>
-      <c r="H23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global cooling efficiency, CESM2 (midlatitude)</t>
-        </is>
-      </c>
-      <c r="B24" s="397">
-        <v>0.236</v>
-      </c>
-      <c r="C24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K per Tg/yr</t>
-        </is>
-      </c>
-      <c r="D24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook tab 6a E10</t>
-        </is>
-      </c>
-      <c r="E24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
-        </is>
-      </c>
-      <c r="F24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate, doi:10.1175/JCLI-D-25-0337.1</t>
-        </is>
-      </c>
-      <c r="G24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value as entered in the workbook. Paper is a stub in precis (0 blocks), so the number could not be read in the source.</t>
-        </is>
-      </c>
-      <c r="H24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global cooling efficiency, E3SMv2 (midlatitude)</t>
-        </is>
-      </c>
-      <c r="B25" s="397">
-        <v>0.0372</v>
-      </c>
-      <c r="C25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K per Tg/yr</t>
-        </is>
-      </c>
-      <c r="D25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook tab 6a E11</t>
-        </is>
-      </c>
-      <c r="E25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
-        </is>
-      </c>
-      <c r="F25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate</t>
-        </is>
-      </c>
-      <c r="G25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">as above</t>
-        </is>
-      </c>
-      <c r="H25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global cooling efficiency, UKESM1.0 (midlatitude)</t>
-        </is>
-      </c>
-      <c r="B26" s="397">
-        <v>0.00754</v>
-      </c>
-      <c r="C26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">K per Tg/yr</t>
-        </is>
-      </c>
-      <c r="D26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook tab 6a E12; CESM2/UKESM1 ratio = 31x</t>
-        </is>
-      </c>
-      <c r="E26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
-        </is>
-      </c>
-      <c r="F26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate</t>
-        </is>
-      </c>
-      <c r="G26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">as above</t>
-        </is>
-      </c>
-      <c r="H26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fraction of emitted aerosol surviving to cloud base</t>
-        </is>
-      </c>
-      <c r="B27" s="397"/>
-      <c r="C27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fraction</t>
-        </is>
-      </c>
-      <c r="D27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook uses 0.3 (0.1-0.5)</t>
-        </is>
-      </c>
-      <c r="E27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3389/fmars.2025.1450175</t>
-        </is>
-      </c>
-      <c r="F27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hernandez-Jaramillo, Kelaher &amp; Harrison, 'A review of plume dispersion and measurement techniques applicable to marine cloud brightening'</t>
-        </is>
-      </c>
-      <c r="G27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The review gives no number. It lists as a priority gap: "estimations of the portion of MCB aerosol reaching cloud base."</t>
-        </is>
-      </c>
-      <c r="H27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Surface temperature sensitivity to forcing (local, reef)</t>
-        </is>
-      </c>
-      <c r="B28" s="397">
-        <v>0.0225</v>
-      </c>
-      <c r="C28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">degC per W/m2</t>
-        </is>
-      </c>
-      <c r="D28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook tab 5a</t>
-        </is>
-      </c>
-      <c r="E28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://gbrrestoration.org/wp-content/uploads/2020/09/T14-Environmental-Modelling-of-Large-Scale-SRM_v3.03-3.pdf</t>
-        </is>
-      </c>
-      <c r="F28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison et al. (2019), RRAP T14 Environmental Modelling of Large-Scale SRM</t>
-        </is>
-      </c>
-      <c r="G28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value as entered in the workbook. PDF cached with no extracted text.</t>
-        </is>
-      </c>
-      <c r="H28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C. Side effects and AMOC</t>
-        </is>
-      </c>
-      <c r="B29" s="401"/>
-      <c r="C29" s="401"/>
-      <c r="D29" s="401"/>
-      <c r="E29" s="401"/>
-      <c r="F29" s="401"/>
-      <c r="G29" s="401"/>
-      <c r="H29" s="401"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global mean precipitation change under +50% CDNC</t>
-        </is>
-      </c>
-      <c r="B30" s="397">
-        <v>-2.35</v>
-      </c>
-      <c r="C30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% (median)</t>
-        </is>
-      </c>
-      <c r="D30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-0.57 to -2.96</t>
-        </is>
-      </c>
-      <c r="E30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="F30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
-        </is>
-      </c>
-      <c r="G30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"a weak but significant precipitation decrease of −2.35 [−0.57 to −2.96] % due to a colder climate, but at low latitudes there is a 1.19 % increase over land."</t>
-        </is>
-      </c>
-      <c r="H30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Low-latitude land precipitation change under +50% CDNC</t>
-        </is>
-      </c>
-      <c r="B31" s="397">
-        <v>1.19</v>
-      </c>
-      <c r="C31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">%</t>
-        </is>
-      </c>
-      <c r="D31" s="397"/>
-      <c r="E31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="F31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stjern et al. (2018), 'Response to marine cloud brightening in a multi-model ensemble' (GeoMIP G4cdnc), published 19 Jan 2018</t>
-        </is>
-      </c>
-      <c r="G31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">same sentence as above</t>
-        </is>
-      </c>
-      <c r="H31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC under regional MCB (3 subtropical oceans, CESM2)</t>
-        </is>
-      </c>
-      <c r="B32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">increase in AMOC index and N. Atlantic gyre mixing depth (magnitude not extracted)</t>
-        </is>
-      </c>
-      <c r="C32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">qualitative</t>
-        </is>
-      </c>
-      <c r="D32" s="397"/>
-      <c r="E32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
-        </is>
-      </c>
-      <c r="F32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa, Hingmire, Singh, Rasch &amp; Mitra (2023), 'Effect of Regional Marine Cloud Brightening Interventions on Climate Tipping Elements', GRL, doi:10.1029/2023GL104314</t>
-        </is>
-      </c>
-      <c r="G32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"increased Atlantic meridional overturning circulation (AMOC) index and North Atlantic gyre mixing depth (Figures 3c and 3h), indicating reduced AMOC collapse risk."</t>
-        </is>
-      </c>
-      <c r="H32" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tipping-element risk under regional MCB (overall)</t>
-        </is>
-      </c>
-      <c r="B33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">reduced overall; some patterns worsen some elements</t>
-        </is>
-      </c>
-      <c r="C33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">qualitative</t>
-        </is>
-      </c>
-      <c r="D33" s="397"/>
-      <c r="E33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
-        </is>
-      </c>
-      <c r="F33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. (2023), GRL</t>
-        </is>
-      </c>
-      <c r="G33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"MCB simulations generally show reduced tipping element risk overall, but certain MCB patterns may exacerbate some tipping element changes"</t>
-        </is>
-      </c>
-      <c r="H33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC under GeoMIP brightening of ocean regions (6 ESMs)</t>
-        </is>
-      </c>
-      <c r="B34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC decreases tied to reduced air-ocean temperature difference and reduced Sept Arctic sea ice; solar dimming more effective than MCB per unit TOA forcing</t>
-        </is>
-      </c>
-      <c r="C34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">qualitative</t>
-        </is>
-      </c>
-      <c r="D34" s="397"/>
-      <c r="E34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-22-4581-2022</t>
-        </is>
-      </c>
-      <c r="F34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xie, Moore, Zhao, Wolovick &amp; Muri (2022), 'Impacts of three types of solar geoengineering on the Atlantic Meridional Overturning Circulation', ACP (published 8 Apr 2022)</t>
-        </is>
-      </c>
-      <c r="G34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"solar dimming is more effective than either marine cloud brightening or stratospheric aerosol injection." Note: the MCB experiment mimics cloud brightening by prescribing ocean brightening, not aerosol microphysics.</t>
-        </is>
-      </c>
-      <c r="H34" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC under regional Arctic solar dimming (proxy, not MCB)</t>
-        </is>
-      </c>
-      <c r="B35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4x stronger local dimming needed to save summer sea ice; MOC reduction and Labrador Sea convection shutdown still possible</t>
-        </is>
-      </c>
-      <c r="C35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">qualitative</t>
-        </is>
-      </c>
-      <c r="D35" s="397"/>
-      <c r="E35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1002/2013GL058731</t>
-        </is>
-      </c>
-      <c r="F35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tilmes, Jahn, Kay, Holland &amp; Lamarque (2014), 'Can regional climate engineering save the summer Arctic sea ice?', GRL, doi:10.1002/2013GL058731</t>
-        </is>
-      </c>
-      <c r="G35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Even with regional Arctic dimming, a reduction in the strength of the oceanic meridional overturning circulation and a shut down of Labrador Sea deep convection are possible."</t>
-        </is>
-      </c>
-      <c r="H35" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC baseline: weakening since ~1950</t>
-        </is>
-      </c>
-      <c r="B36" s="397">
-        <v>3</v>
-      </c>
-      <c r="C36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sv (+/- 1)</t>
-        </is>
-      </c>
-      <c r="D36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC currently 'weakest in over a millennium' per proxy records cited therein</t>
-        </is>
-      </c>
-      <c r="E36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1126/sciadv.adk1189</t>
-        </is>
-      </c>
-      <c r="F36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">van Westen, Kliphuis &amp; Dijkstra (2024), 'Physics-based early warning signal shows that AMOC is on tipping course', Sci. Adv., doi:10.1126/sciadv.adk1189</t>
-        </is>
-      </c>
-      <c r="G36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"indicates that the AMOC weakened by 3 ± 1 Sv since about 1950."</t>
-        </is>
-      </c>
-      <c r="H36" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fisheries / marine ecosystem effect (magnitude)</t>
-        </is>
-      </c>
-      <c r="B37" s="397"/>
-      <c r="C37" s="397"/>
-      <c r="D37" s="397"/>
-      <c r="E37" s="397"/>
-      <c r="F37" s="397"/>
-      <c r="G37" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Side-effects strand has no ingested papers yet.</t>
-        </is>
-      </c>
-      <c r="H37" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salt deposition on land (magnitude)</t>
-        </is>
-      </c>
-      <c r="B38" s="397"/>
-      <c r="C38" s="397"/>
-      <c r="D38" s="397"/>
-      <c r="E38" s="397"/>
-      <c r="F38" s="397"/>
-      <c r="G38" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Side-effects strand has no ingested papers yet.</t>
-        </is>
-      </c>
-      <c r="H38" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dollar value of maintaining AMOC</t>
-        </is>
-      </c>
-      <c r="B39" s="397"/>
-      <c r="C39" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$</t>
-        </is>
-      </c>
-      <c r="D39" s="397"/>
-      <c r="E39" s="397"/>
-      <c r="F39" s="397"/>
-      <c r="G39" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No economic valuation found among the 20 linked AMOC papers read at title/abstract level.</t>
-        </is>
-      </c>
-      <c r="H39" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">D. MCB cost estimates in the literature (Perplexity only; secondary, not primary)</t>
-        </is>
-      </c>
-      <c r="B40" s="401"/>
-      <c r="C40" s="401"/>
-      <c r="D40" s="401"/>
-      <c r="E40" s="401"/>
-      <c r="F40" s="401"/>
-      <c r="G40" s="401"/>
-      <c r="H40" s="401"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MCB deployment cost, general literature (origin of the '~$10B/yr' framing)</t>
-        </is>
-      </c>
-      <c r="B41" s="397">
-        <v>10</v>
-      </c>
-      <c r="C41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$B/yr</t>
-        </is>
-      </c>
-      <c r="D41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">'poorly characterized'</t>
-        </is>
-      </c>
-      <c r="E41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6784395/</t>
-        </is>
-      </c>
-      <c r="F41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer citing one review (PMC6784395); review text not read</t>
-        </is>
-      </c>
-      <c r="G41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"One review reports that MCB deployment costs are poorly characterized but might be around $10 billion per year."</t>
-        </is>
-      </c>
-      <c r="H41" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NASEM logistics estimate, Arctic MCB</t>
-        </is>
-      </c>
-      <c r="B42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 per week for 0.01 W/m2</t>
-        </is>
-      </c>
-      <c r="C42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$M/week per 0.01 W/m2</t>
-        </is>
-      </c>
-      <c r="D42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity annualises to ~$26B per W/m2-yr</t>
-        </is>
-      </c>
-      <c r="E42" s="397"/>
-      <c r="F42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer; underlying NASEM text not read</t>
-        </is>
-      </c>
-      <c r="G42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Approximately $5 million per week to produce 0.01 W/m² of forcing."</t>
-        </is>
-      </c>
-      <c r="H42" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regional Arctic MCB fleet</t>
-        </is>
-      </c>
-      <c r="B43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">500-1,000 vessels; capex up to GBP 40bn; ~GBP 10bn/yr running</t>
-        </is>
-      </c>
-      <c r="C43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mixed</t>
-        </is>
-      </c>
-      <c r="D43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">media/interview estimate</t>
-        </is>
-      </c>
-      <c r="E43" s="397"/>
-      <c r="F43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer; underlying source not read</t>
-        </is>
-      </c>
-      <c r="G43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"500–1,000 vessels, with capital cost up to £40bn and continuation costs around £10bn/year." Currency left as reported (GBP), not converted.</t>
-        </is>
-      </c>
-      <c r="H43" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Airborne MCB concept</t>
-        </is>
-      </c>
-      <c r="B44" s="397">
-        <v>40</v>
-      </c>
-      <c r="C44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$bn/yr</t>
-        </is>
-      </c>
-      <c r="D44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">autonomous-ship electricity alone ~$41bn/yr</t>
-        </is>
-      </c>
-      <c r="E44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1088/2515-7620/ad2f71</t>
-        </is>
-      </c>
-      <c r="F44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer citing iopscience 10.1088/2515-7620/ad2f71; not read</t>
-        </is>
-      </c>
-      <c r="G44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Estimated operational cost around $40bn/year"</t>
-        </is>
-      </c>
-      <c r="H44" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E. Damage per degree of warming (feeds the workbook's value-per-K)</t>
-        </is>
-      </c>
-      <c r="B45" s="401"/>
-      <c r="C45" s="401"/>
-      <c r="D45" s="401"/>
-      <c r="E45" s="401"/>
-      <c r="F45" s="401"/>
-      <c r="G45" s="401"/>
-      <c r="H45" s="401"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Damage, low (Nordhaus DICE-2016R)</t>
-        </is>
-      </c>
-      <c r="B46" s="397">
-        <v>0.6</v>
-      </c>
-      <c r="C46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% GDP per degC</t>
-        </is>
-      </c>
-      <c r="D46" s="397"/>
-      <c r="E46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3386/w22933</t>
-        </is>
-      </c>
-      <c r="F46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nordhaus (2016), NBER w22933 (DICE-2016R), as cited in workbook tab 6a G43</t>
-        </is>
-      </c>
-      <c r="G46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value as entered in the workbook. Source not ingested.</t>
-        </is>
-      </c>
-      <c r="H46" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Damage, central (Burke, Hsiang &amp; Miguel 2015)</t>
-        </is>
-      </c>
-      <c r="B47" s="397">
-        <v>3.3</v>
-      </c>
-      <c r="C47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% GDP per degC</t>
-        </is>
-      </c>
-      <c r="D47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workbook derives from ~23% at ~3.7 degC</t>
-        </is>
-      </c>
-      <c r="E47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
-        </is>
-      </c>
-      <c r="F47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Burke, Hsiang &amp; Miguel (2015), Nature 527:235</t>
-        </is>
-      </c>
-      <c r="G47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value as entered in the workbook. Paper is a stub in precis (0 blocks); 3.3%/degC is the workbook's own conversion.</t>
-        </is>
-      </c>
-      <c r="H47" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Burke et al. 2015: global income loss by 2100, unmitigated</t>
-        </is>
-      </c>
-      <c r="B48" s="397">
-        <v>23</v>
-      </c>
-      <c r="C48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% lower income</t>
-        </is>
-      </c>
-      <c r="D48" s="397"/>
-      <c r="E48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
-        </is>
-      </c>
-      <c r="F48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer on Burke et al., doi:10.1038/nature15725</t>
-        </is>
-      </c>
-      <c r="G48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"approximately 23% lower global average income by 2100"</t>
-        </is>
-      </c>
-      <c r="H48" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Damage, high (Bilal &amp; Kanzig 2024)</t>
-        </is>
-      </c>
-      <c r="B49" s="397">
-        <v>12</v>
-      </c>
-      <c r="C49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% GDP per degC</t>
-        </is>
-      </c>
-      <c r="D49" s="397"/>
-      <c r="E49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3386/w32450</t>
-        </is>
-      </c>
-      <c r="F49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bilal &amp; Kanzig (2024), NBER w32450, as cited in workbook tab 6a G45</t>
-        </is>
-      </c>
-      <c r="G49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value as entered in the workbook. Not ingested; Perplexity states it found no source exposing the paper's exact coefficient.</t>
-        </is>
-      </c>
-      <c r="H49" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub; unverified</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kotz, Levermann &amp; Wenz 2024: world income loss by 2050</t>
-        </is>
-      </c>
-      <c r="B50" s="397">
-        <v>19</v>
-      </c>
-      <c r="C50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">% lower income</t>
-        </is>
-      </c>
-      <c r="D50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11-29% likely range</t>
-        </is>
-      </c>
-      <c r="E50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/s41586-024-07219-0</t>
-        </is>
-      </c>
-      <c r="F50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer on Kotz et al., Nature, doi:10.1038/s41586-024-07219-0</t>
-        </is>
-      </c>
-      <c r="G50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Projected 19% lower world income by 2050, with a likely range of 11–29%" (a level, not a per-degC coefficient; Perplexity notes it has been challenged).</t>
-        </is>
-      </c>
-      <c r="H50" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Share of hail losses that scales with temperature</t>
-        </is>
-      </c>
-      <c r="B51" s="397"/>
-      <c r="C51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">%</t>
-        </is>
-      </c>
-      <c r="D51" s="397"/>
-      <c r="E51" s="397"/>
-      <c r="F51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perplexity answer</t>
-        </is>
-      </c>
-      <c r="G51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Hail ... Not sourced." Perplexity found no defensible figure.</t>
-        </is>
-      </c>
-      <c r="H51" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F. Benefit side: 2026 European severe convective storm (SCS) insured losses</t>
-        </is>
-      </c>
-      <c r="B52" s="401"/>
-      <c r="C52" s="401"/>
-      <c r="D52" s="401"/>
-      <c r="E52" s="401"/>
-      <c r="F52" s="401"/>
-      <c r="G52" s="401"/>
-      <c r="H52" s="401"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SCS 'Cerry', 13-19 Jul 2026 (DE/FR/CH/IT): second estimate</t>
-        </is>
-      </c>
-      <c r="B53" s="397">
-        <v>2806.0</v>
-      </c>
-      <c r="C53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR m</t>
-        </is>
-      </c>
-      <c r="D53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">initial estimate 2,186; provisional</t>
-        </is>
-      </c>
-      <c r="E53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026</t>
-        </is>
-      </c>
-      <c r="F53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PERILS AG industry loss estimate (Zurich), released 20 Oct 2026, perils.org</t>
-        </is>
-      </c>
-      <c r="G53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"PERILS’ second estimate of the insurance market loss is EUR 2,806 million. This compares to the initial loss estimate of EUR 2,186 million."</t>
-        </is>
-      </c>
-      <c r="H53" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SCS 'Raphaela', 26-28 Aug 2026 (FR/DE/CH/IT): first estimate</t>
-        </is>
-      </c>
-      <c r="B54" s="397">
-        <v>3296.0</v>
-      </c>
-      <c r="C54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR m</t>
-        </is>
-      </c>
-      <c r="D54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">provisional; large hail, wind, flash flood</t>
-        </is>
-      </c>
-      <c r="E54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
-        </is>
-      </c>
-      <c r="F54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PERILS AG industry loss estimate (Zurich), released 19 Oct 2026, perils.org</t>
-        </is>
-      </c>
-      <c r="G54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"PERILS’ initial estimate of the insurance market loss is EUR 3,296 million. Losses were the result of large hail, high winds and flash flooding."</t>
-        </is>
-      </c>
-      <c r="H54" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sum of the two PERILS estimates (derived)</t>
-        </is>
-      </c>
-      <c r="B55" s="397">
-        <v>6102.0</v>
-      </c>
-      <c r="C55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR m</t>
-        </is>
-      </c>
-      <c r="D55" s="397"/>
-      <c r="E55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
-        </is>
-      </c>
-      <c r="F55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">arithmetic</t>
-        </is>
-      </c>
-      <c r="G55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2,806 + 3,296 = 6,102 (EUR 6.1B). Both estimates are provisional and PERILS says updates follow.</t>
-        </is>
-      </c>
-      <c r="H55" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Earlier vintage sum (Cerry initial + Raphaela)</t>
-        </is>
-      </c>
-      <c r="B56" s="397">
-        <v>5482.0</v>
-      </c>
-      <c r="C56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR m</t>
-        </is>
-      </c>
-      <c r="D56" s="397"/>
-      <c r="E56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
-        </is>
-      </c>
-      <c r="F56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">arithmetic</t>
-        </is>
-      </c>
-      <c r="G56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2,186 + 3,296 = 5,482. This is the strand's earlier '~EUR 5.5B'; superseded by the 6,102 above.</t>
-        </is>
-      </c>
-      <c r="H56" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cerry second estimate in USD</t>
-        </is>
-      </c>
-      <c r="B57" s="397">
-        <v>3208.7</v>
-      </c>
-      <c r="C57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m</t>
-        </is>
-      </c>
-      <c r="D57" s="397"/>
-      <c r="E57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://api.frankfurter.app</t>
-        </is>
-      </c>
-      <c r="F57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand conversion</t>
-        </is>
-      </c>
-      <c r="G57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2,806 x 1.1435. EUR/USD 1.1435, ECB reference rate via api.frankfurter.app, rate date 2026-07-17 (last ECB publication on/before event end 2026-07-19, a Sunday).</t>
-        </is>
-      </c>
-      <c r="H57" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Raphaela first estimate in USD</t>
-        </is>
-      </c>
-      <c r="B58" s="397">
-        <v>3837.5</v>
-      </c>
-      <c r="C58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m</t>
-        </is>
-      </c>
-      <c r="D58" s="397"/>
-      <c r="E58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
-        </is>
-      </c>
-      <c r="F58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand conversion</t>
-        </is>
-      </c>
-      <c r="G58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3,296 x 1.1643. EUR/USD 1.1643, ECB reference rate via api.frankfurter.app, rate date 2026-08-28 (event end date).</t>
-        </is>
-      </c>
-      <c r="H58" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sum of the two events in USD (event-date rates)</t>
-        </is>
-      </c>
-      <c r="B59" s="397">
-        <v>7046.2</v>
-      </c>
-      <c r="C59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m</t>
-        </is>
-      </c>
-      <c r="D59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6843.4 at the release-date rate 1.1215 (ECB 2026-10-20)</t>
-        </is>
-      </c>
-      <c r="E59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
-        </is>
-      </c>
-      <c r="F59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand conversion</t>
-        </is>
-      </c>
-      <c r="G59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3208.7 + 3837.5. Release-date sensitivity: 6,102 x 1.1215 = 6843.4.</t>
-        </is>
-      </c>
-      <c r="H59" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Europe SCS insured losses, 9M 2026 (Gallagher Re)</t>
-        </is>
-      </c>
-      <c r="B60" s="397">
-        <v>9000</v>
-      </c>
-      <c r="C60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m (at least)</t>
-        </is>
-      </c>
-      <c r="D60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">includes USD 3.8B for the late-August outbreak</t>
-        </is>
-      </c>
-      <c r="E60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
-        </is>
-      </c>
-      <c r="F60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinsurance News, 21 Oct 2026, reporting Gallagher Re Q3 2026 Natural Catastrophe and Climate Report (the primary Gallagher Re report page has no extractable text)</t>
-        </is>
-      </c>
-      <c r="G60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"In Europe, insured losses associated with severe convective storms reached at least USD $9 billion, according to Gallagher Re. This included USD $3.8 billion in losses resulting from an outbreak in late August." Secondary relay.</t>
-        </is>
-      </c>
-      <c r="H60" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gallagher late-August Europe SCS vs PERILS Raphaela converted</t>
-        </is>
-      </c>
-      <c r="B61" s="397">
-        <v>3800</v>
-      </c>
-      <c r="C61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m</t>
-        </is>
-      </c>
-      <c r="D61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PERILS Raphaela converted = 3837.5</t>
-        </is>
-      </c>
-      <c r="E61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
-        </is>
-      </c>
-      <c r="F61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cross-check</t>
-        </is>
-      </c>
-      <c r="G61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gallagher 3.8B USD against 3,296 EUR x 1.1643: consistent at 2 significant figures. Different insurer scopes.</t>
-        </is>
-      </c>
-      <c r="H61" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">US SCS insured losses, 9M 2026 (context)</t>
-        </is>
-      </c>
-      <c r="B62" s="397">
-        <v>43000</v>
-      </c>
-      <c r="C62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">USD m (at least)</t>
-        </is>
-      </c>
-      <c r="D62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">global insured nat cat: USD 92B</t>
-        </is>
-      </c>
-      <c r="E62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
-        </is>
-      </c>
-      <c r="F62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinsurance News on Gallagher Re</t>
-        </is>
-      </c>
-      <c r="G62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"insured losses from these storms in the United States reached at least USD $43 billion by the end of the third quarter."</t>
-        </is>
-      </c>
-      <c r="H62" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A52:H52"/>
-  </mergeCells>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-  </sheetPr>
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="52" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="52" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="48" customHeight="1">
-      <c r="A1" s="400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Reads the workbook's figures against the Survey tab. Workbook numbers were read from the file unchanged; no workbook formula or value was edited. Literature notes sit in an adjacent column on the tabs themselves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Item</t>
-        </is>
-      </c>
-      <c r="B3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook value</t>
-        </is>
-      </c>
-      <c r="C3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook location</t>
-        </is>
-      </c>
-      <c r="D3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Survey comparison</t>
-        </is>
-      </c>
-      <c r="E3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source link</t>
-        </is>
-      </c>
-      <c r="F3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reading</t>
-        </is>
-      </c>
-      <c r="G3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flag</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BLUF: (1) The workbook contains no '~$10B/yr' figure; its cost anchors are $21.4M/yr per dedicated vessel, $9.3M/yr per piggyback ship and $175B-$18T/yr for 1 K of global cooling. (2) Its nozzle power (512 W) and output (1.73e12 particles/s) match the Harrison et al. 2025 paper held in precis, but the 150 nm design size is not what that nozzle makes (count median 49.5 nm). (3) Its tonnage-per-K spread (31x) comes from a J. Climate paper that is a stub in precis; the full-text preprint by the same group gives 13x for equal forcing. (4) The damage-per-K band (0.6/3.3/12 % of GDP) rests on sources with no text in precis. (5) The two 2026 EU storm events (about USD 7.0B insured, hand-converted) are 329 dedicated vessel-years or 761 piggyback ship-years of Tito's cost, and 0.04%-4.0% of his per-K annual cost; hail and AMOC bear on the benefit side only as a scale cross-check and a model-dependent caveat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. The '~$10B/yr' framing</t>
-        </is>
-      </c>
-      <c r="B5" s="401"/>
-      <c r="C5" s="401"/>
-      <c r="D5" s="401"/>
-      <c r="E5" s="401"/>
-      <c r="F5" s="401"/>
-      <c r="G5" s="401"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">'~$10B/yr' deployment cost</t>
-        </is>
-      </c>
-      <c r="B6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">does NOT appear</t>
-        </is>
-      </c>
-      <c r="C6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">searched all 17 tabs: no text match and no numeric cell between 9e9 and 1.1e10</t>
-        </is>
-      </c>
-      <c r="D6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The framing traces to a Perplexity summary of one review ('might be around $10 billion per year'), not to the workbook.</t>
-        </is>
-      </c>
-      <c r="E6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://pmc.ncbi.nlm.nih.gov/articles/PMC6784395/</t>
-        </is>
-      </c>
-      <c r="F6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nearest workbook number: one piggyback ship at $9.26M/yr (tab 3b), 1000x smaller. Per-K cost $175B-$18T/yr is 17x to 1,800x the $10B. Comparisons below use the workbook's own costs.</t>
-        </is>
-      </c>
-      <c r="G6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">perplexity-only</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2. Workbook cost figures against the survey</t>
-        </is>
-      </c>
-      <c r="B7" s="401"/>
-      <c r="C7" s="401"/>
-      <c r="D7" s="401"/>
-      <c r="E7" s="401"/>
-      <c r="F7" s="401"/>
-      <c r="G7" s="401"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Levelized cost, dedicated vessel</t>
-        </is>
-      </c>
-      <c r="B8" s="397">
-        <v>54048</v>
-      </c>
-      <c r="C8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3a C13 ($/t); annual $21,389,498 (3a B13)</t>
-        </is>
-      </c>
-      <c r="D8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No independent $/t exists in the survey. Inputs: nozzle power 513 W derived vs 512 W used, particle rate 1.73e12/s identical.</t>
-        </is>
-      </c>
-      <c r="E8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="F8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Energy input confirmed by source. Vessel price, fuel, compressor $/kW, survival 0.3 have no source in precis. Nozzle price $50 cited to RRAP CS-07 (no text).</t>
-        </is>
-      </c>
-      <c r="G8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified; no-source; stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Levelized cost, piggyback (3b)</t>
-        </is>
-      </c>
-      <c r="B9" s="397">
-        <v>21674</v>
-      </c>
-      <c r="C9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 B7 ($/t); $9,259,922/yr (4 C7)</t>
-        </is>
-      </c>
-      <c r="D9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Deck-slot rent $2M, technicians, 4.5 MW gensets: no survey source.</t>
-        </is>
-      </c>
-      <c r="E9" s="397"/>
-      <c r="F9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No source in precis for the scenario-specific lines.</t>
-        </is>
-      </c>
-      <c r="G9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Levelized cost, fixed platform (3c)</t>
-        </is>
-      </c>
-      <c r="B10" s="397">
-        <v>14633</v>
-      </c>
-      <c r="C10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 B8 ($/t); $5,791,171/yr (4 C8)</t>
-        </is>
-      </c>
-      <c r="D10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Platform $3M, siting, mooring, shore power: no survey source.</t>
-        </is>
-      </c>
-      <c r="E10" s="397"/>
-      <c r="F10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">As above.</t>
-        </is>
-      </c>
-      <c r="G10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Levelized cost, stationary vessel (3d)</t>
-        </is>
-      </c>
-      <c r="B11" s="397">
-        <v>49341</v>
-      </c>
-      <c r="C11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4 B9 ($/t); $19,526,858/yr (4 C9)</t>
-        </is>
-      </c>
-      <c r="D11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No survey source.</t>
-        </is>
-      </c>
-      <c r="E11" s="397"/>
-      <c r="F11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">As above.</t>
-        </is>
-      </c>
-      <c r="G11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Particle size at design point</t>
-        </is>
-      </c>
-      <c r="B12" s="397">
-        <v>150</v>
-      </c>
-      <c r="C12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a B20 (nm)</t>
-        </is>
-      </c>
-      <c r="D12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nozzle count median diameter 49.5 nm, GSD 2.01. ESMs emit 28.1-72.5 nm (preprint); workbook restates tonnage to 150 nm via (150/d)^3.</t>
-        </is>
-      </c>
-      <c r="E12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D  https://doi.org/10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="F12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Open question for Tito: how a nozzle with CMD 49.5 nm yields the 150 nm design basis (the cubic size correction in 6a F34:F37 moves tonnage by factors of 0.75-1.02 only).</t>
-        </is>
-      </c>
-      <c r="G12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Climate-model spread, K per Tg/yr (CESM2 / UKESM1)</t>
-        </is>
-      </c>
-      <c r="B13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31x (0.236 vs 0.00754)</t>
-        </is>
-      </c>
-      <c r="C13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a E10, E12</t>
-        </is>
-      </c>
-      <c r="D13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Preprint, equal -2 W/m2: emissions 7-93 Tg/yr = 13x. GeoMIP G4cdnc ERF for the same CDNC change: -0.6 to -2.5 W/m2 = 4.2x.</t>
-        </is>
-      </c>
-      <c r="E13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460  https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="F13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workbook spread is the J. Climate paper's (stub, cannot be checked). The two full-text sources give a smaller spread.</t>
-        </is>
-      </c>
-      <c r="G13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value of 1 K for a year, low</t>
-        </is>
-      </c>
-      <c r="B14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$660B</t>
-        </is>
-      </c>
-      <c r="C14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D20 (0.6% x $110T)</t>
-        </is>
-      </c>
-      <c r="D14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nordhaus DICE source not ingested.</t>
-        </is>
-      </c>
-      <c r="E14" s="397"/>
-      <c r="F14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value is arithmetic on a GDP share with no source text.</t>
-        </is>
-      </c>
-      <c r="G14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value of 1 K for a year, central</t>
-        </is>
-      </c>
-      <c r="B15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$3,630B</t>
-        </is>
-      </c>
-      <c r="C15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D21 (3.3% x $110T)</t>
-        </is>
-      </c>
-      <c r="D15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Burke 2015 is a stub; the 3.3%/degC is the workbook's conversion of ~23% at ~3.7 degC. Perplexity gives 23% by 2100 (not a per-degC rate).</t>
-        </is>
-      </c>
-      <c r="E15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
-        </is>
-      </c>
-      <c r="F15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Central case has no readable source in precis.</t>
-        </is>
-      </c>
-      <c r="G15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value of 1 K for a year, high</t>
-        </is>
-      </c>
-      <c r="B16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$13,200B</t>
-        </is>
-      </c>
-      <c r="C16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D22 (12% x $110T)</t>
-        </is>
-      </c>
-      <c r="D16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bilal &amp; Kanzig 2024 not ingested; Perplexity could not find the coefficient.</t>
-        </is>
-      </c>
-      <c r="E16" s="397"/>
-      <c r="F16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Treat as unverified.</t>
-        </is>
-      </c>
-      <c r="G16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub; unverified</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCR, dedicated vessel, 4 model cases</t>
-        </is>
-      </c>
-      <c r="B17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.64 / 8.30 / 0.877 / 0.202</t>
-        </is>
-      </c>
-      <c r="C17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D29:D32 (CESM2, CESM2-Ghosh, E3SMv2, UKESM1); costs $0.78T / $0.44T / $4.14T / $17.97T per year</t>
-        </is>
-      </c>
-      <c r="D17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Numerator is the central $3,630B (stub-sourced); denominator spread is the 31x tonnage spread (stub-sourced).</t>
-        </is>
-      </c>
-      <c r="E17" s="397"/>
-      <c r="F17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Both halves of the ratio rest on sources not readable in precis. The 6b header says '$B/yr' but cells hold raw dollars.</t>
-        </is>
-      </c>
-      <c r="G17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BCR, piggyback, 4 model cases</t>
-        </is>
-      </c>
-      <c r="B18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11.6 / 20.7 / 2.19 / 0.504</t>
-        </is>
-      </c>
-      <c r="C18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6c D38:D41; costs $0.31T / $0.18T / $1.66T / $7.21T per year</t>
-        </is>
-      </c>
-      <c r="D18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Same as above.</t>
-        </is>
-      </c>
-      <c r="E18" s="397"/>
-      <c r="F18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Same as above.</t>
-        </is>
-      </c>
-      <c r="G18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cooling from one dedicated vessel (consistency check)</t>
-        </is>
-      </c>
-      <c r="B19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.74e-05 K</t>
-        </is>
-      </c>
-      <c r="C19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">396 t/yr (3a B22) / 14.46 Mt/yr (6b D10, CESM2)</t>
-        </is>
-      </c>
-      <c r="D19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value at central damage = $99.4M against $21.4M cost = BCR 4.64, equal to 6b D29.</t>
-        </is>
-      </c>
-      <c r="E19" s="397"/>
-      <c r="F19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internal arithmetic only; confirms 6b is consistent with 3a.</t>
-        </is>
-      </c>
-      <c r="G19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3. 2026 EU storm losses against Tito's per-vessel and per-K costs (not against $10B)</t>
-        </is>
-      </c>
-      <c r="B20" s="401"/>
-      <c r="C20" s="401"/>
-      <c r="D20" s="401"/>
-      <c r="E20" s="401"/>
-      <c r="F20" s="401"/>
-      <c r="G20" s="401"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two EU events, insured, in USD</t>
-        </is>
-      </c>
-      <c r="B21" s="397">
-        <v>7046.2</v>
-      </c>
-      <c r="C21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">survey F (USD m)</t>
-        </is>
-      </c>
-      <c r="D21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PERILS EUR 2,806m + 3,296m = EUR 6,102m, converted at event-date ECB rates</t>
-        </is>
-      </c>
-      <c r="E21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026  https://api.frankfurter.app</t>
-        </is>
-      </c>
-      <c r="F21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR/USD 1.1435, ECB reference rate via api.frankfurter.app, rate date 2026-07-17 (last ECB publication on/before event end 2026-07-19, a Sunday); EUR/USD 1.1643, ECB reference rate via api.frankfurter.app, rate date 2026-08-28 (event end date).</t>
-        </is>
-      </c>
-      <c r="G21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">... in dedicated vessel-years</t>
-        </is>
-      </c>
-      <c r="B22" s="397">
-        <v>329.4</v>
-      </c>
-      <c r="C22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vs 3a B13 $21,389,498/yr</t>
-        </is>
-      </c>
-      <c r="D22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">329.4 vessel-years; one vessel-year = 0.30% of the two events</t>
-        </is>
-      </c>
-      <c r="E22" s="397"/>
-      <c r="F22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Insured loss of two events divided by one vessel's annual levelized cost.</t>
-        </is>
-      </c>
-      <c r="G22" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">... in piggyback ship-years</t>
-        </is>
-      </c>
-      <c r="B23" s="397">
-        <v>760.9</v>
-      </c>
-      <c r="C23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vs 4 C7 $9,259,922/yr</t>
-        </is>
-      </c>
-      <c r="D23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">760.9 ship-years; one ship-year = 0.13% of the two events</t>
-        </is>
-      </c>
-      <c r="E23" s="397"/>
-      <c r="F23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">As above.</t>
-        </is>
-      </c>
-      <c r="G23" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">... as share of dedicated-vessel cost of 1 K (4 cases)</t>
-        </is>
-      </c>
-      <c r="B24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.902% / 1.61% / 0.17% / 0.0392%</t>
-        </is>
-      </c>
-      <c r="C24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b E10:E13</t>
-        </is>
-      </c>
-      <c r="D24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CESM2 / CESM2-Ghosh / E3SMv2 / UKESM1</t>
-        </is>
-      </c>
-      <c r="E24" s="397"/>
-      <c r="F24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two events alone pay 0.04%-0.9% of a year of 1 K cooling.</t>
-        </is>
-      </c>
-      <c r="G24" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">... as share of piggyback cost of 1 K (4 cases)</t>
-        </is>
-      </c>
-      <c r="B25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.25% / 4.02% / 0.425% / 0.0978%</t>
-        </is>
-      </c>
-      <c r="C25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6c E18:E21</t>
-        </is>
-      </c>
-      <c r="D25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CESM2 / CESM2-Ghosh / E3SMv2 / UKESM1</t>
-        </is>
-      </c>
-      <c r="E25" s="397"/>
-      <c r="F25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Two events alone pay 0.1%-4.0% of a year of 1 K cooling.</t>
-        </is>
-      </c>
-      <c r="G25" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">... as share of the workbook's value of 1 K-yr (low/central/high)</t>
-        </is>
-      </c>
-      <c r="B26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.07% / 0.194% / 0.0534%</t>
-        </is>
-      </c>
-      <c r="C26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D20:D22</t>
-        </is>
-      </c>
-      <c r="D26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$660B / $3,630B / $13,200B</t>
-        </is>
-      </c>
-      <c r="E26" s="397"/>
-      <c r="F26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Insured storm losses are a small slice of the damage-function value.</t>
-        </is>
-      </c>
-      <c r="G26" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gallagher Re: Europe SCS 9M 2026, at least USD 9B</t>
-        </is>
-      </c>
-      <c r="B27" s="397">
-        <v>9000</v>
-      </c>
-      <c r="C27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">survey F (USD m)</t>
-        </is>
-      </c>
-      <c r="D27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">421 dedicated vessel-years; 972 piggyback ship-years</t>
-        </is>
-      </c>
-      <c r="E27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
-        </is>
-      </c>
-      <c r="F27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Whole-year-to-date Europe, USD as reported (no conversion). Includes the late-August USD 3.8B outbreak, so it overlaps the PERILS sum; do not add them.</t>
-        </is>
-      </c>
-      <c r="G27" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Limits of this comparison: two events in one season are not an annual loss; insured loss is below economic loss; PERILS estimates are provisional (updates follow); and no source in precis says how much of this hail loss 1 K of marine cloud brightening would avoid (Perplexity: share of hail loss that scales with temperature 'Not sourced'). The storm losses are therefore context for scale, not a benefit line to add to 6b/6c, and would partly overlap the damage-function value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4. Where hail and AMOC bear on what the workbook computes</t>
-        </is>
-      </c>
-      <c r="B29" s="401"/>
-      <c r="C29" s="401"/>
-      <c r="D29" s="401"/>
-      <c r="E29" s="401"/>
-      <c r="F29" s="401"/>
-      <c r="G29" s="401"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hail / severe convective storm insured loss vs the damage-function value</t>
-        </is>
-      </c>
-      <c r="B30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EUR 6,102m (about USD 7046m) for two 2026 events</t>
-        </is>
-      </c>
-      <c r="C30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b D20:D22 value of 1 K-yr</t>
-        </is>
-      </c>
-      <c r="D30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The workbook values cooling through GDP-wide damage per degC, which already contains storm damage. Two events are 0.194% of the central $3,630B/K-yr: a scale cross-check, not an extra line to add.</t>
-        </is>
-      </c>
-      <c r="E30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news/eur-2-806m-perils-releases-second-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-mid-july-2026  https://www.perils.org/news/eur-3-296m-first-perils-industry-loss-estimate-for-the-severe-convective-storms-in-europe-of-late-august-2026</t>
-        </is>
-      </c>
-      <c r="F30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No source in precis gives the hail share of the damage function or the hail loss avoided per K.</t>
-        </is>
-      </c>
-      <c r="G30" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hand-FX</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AMOC</t>
-        </is>
-      </c>
-      <c r="B31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">qualitative only</t>
-        </is>
-      </c>
-      <c r="C31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b/6c benefit side (value of cooling)</t>
-        </is>
-      </c>
-      <c r="D31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Whether the cooling benefit includes reduced AMOC-collapse risk is model-dependent: CESM2 regional MCB raises the AMOC index (Hirasawa 2023); GeoMIP ocean brightening still lowers AMOC (Xie 2022).</t>
-        </is>
-      </c>
-      <c r="E31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314  https://doi.org/10.5194/acp-22-4581-2022</t>
-        </is>
-      </c>
-      <c r="F31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No dollar value found, so no number is proposed for the workbook.</t>
-        </is>
-      </c>
-      <c r="G31" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no-source</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flag legend</t>
-        </is>
-      </c>
-      <c r="B32" s="401"/>
-      <c r="C32" s="401"/>
-      <c r="D32" s="401"/>
-      <c r="E32" s="401"/>
-      <c r="F32" s="401"/>
-      <c r="G32" s="401"/>
-    </row>
-    <row r="33" ht="45" customHeight="1">
-      <c r="A33" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stub = source paper/report has no full text in precis; perplexity-only = only source is a Perplexity ref; hand-FX = currency conversion done by hand with the ECB rate (date and rate recorded); unverified = quote not found in source text; no-source = cell left empty; verified = value and quote read in text held in precis (or arithmetic on such values). Workbook cell values were read from the file with a data-only loader.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A32:G32"/>
-    <mergeCell ref="A33:G33"/>
-  </mergeCells>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="40" style="167" customWidth="1"/>
@@ -19105,9 +15932,7 @@
     <col min="3" max="3" width="14" style="167" customWidth="1"/>
     <col min="4" max="4" width="68" style="167" customWidth="1"/>
     <col min="5" max="5" width="55" style="167" customWidth="1"/>
-    <col min="6" max="9" width="8.6640625" style="167"/>
-    <col min="10" max="10" width="120" style="167" customWidth="1"/>
-    <col min="11" max="16384" width="8.6640625" style="167"/>
+    <col min="6" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -19144,7 +15969,7 @@
       <c r="E6" s="168"/>
       <c r="F6" s="168"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="181" t="s">
         <v>13</v>
       </c>
@@ -19161,13 +15986,8 @@
         <v>17</v>
       </c>
       <c r="F7" s="168"/>
-      <c r="J7" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="117" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="8" spans="1:7" ht="117" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="183" t="s">
         <v>18</v>
       </c>
@@ -19184,13 +16004,8 @@
         <v>788</v>
       </c>
       <c r="F8" s="168"/>
-      <c r="J8" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: 1.73e12 particles/s for the best nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="9" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="183" t="s">
         <v>21</v>
       </c>
@@ -19205,13 +16020,8 @@
         <v>788</v>
       </c>
       <c r="F9" s="168"/>
-      <c r="J9" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: 71% of particles fall in 30-1000 nm (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="10" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="183" t="s">
         <v>23</v>
       </c>
@@ -19228,11 +16038,6 @@
         <v>789</v>
       </c>
       <c r="F10" s="168"/>
-      <c r="J10" s="403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFLICT: lit count median dry diameter 49.5 nm, GSD 2.01, ~94% of particles below 200 nm for the best nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D); ESMs emit median modal radii of 28.1-72.5 nm (Hirasawa preprint, https://doi.org/10.5194/egusphere-2026-5460). Workbook uses 150 nm.</t>
-        </is>
-      </c>
     </row>
     <row r="11" spans="1:7" ht="41.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="183" t="s">
@@ -19321,7 +16126,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="17" ht="66" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:9" ht="66" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="183" t="s">
         <v>34</v>
       </c>
@@ -19347,11 +16152,6 @@
       </c>
       <c r="I17" s="185" t="s">
         <v>884</v>
-      </c>
-      <c r="J17" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: 417.4 kW for 814 nozzles = 513 W per nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D); ARIEL prototype 100 nozzles ~55 kW (~550 W each). Workbook 512 W matches.</t>
-        </is>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
@@ -19440,7 +16240,7 @@
       <c r="E22" s="168"/>
       <c r="F22" s="168"/>
     </row>
-    <row r="23" ht="79" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:9" ht="79" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="183" t="s">
         <v>40</v>
       </c>
@@ -19457,11 +16257,6 @@
         <v>791</v>
       </c>
       <c r="F23" s="168"/>
-      <c r="J23" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: 0.41 mL/s seawater + 0.3 L/s air per nozzle (Harrison 2025, https://doi.org/10.1039/D5EA00073D). Matches the workbook.</t>
-        </is>
-      </c>
     </row>
     <row r="24" spans="1:9" ht="26" x14ac:dyDescent="0.15">
       <c r="A24" s="183" t="s">
@@ -19497,7 +16292,7 @@
       <c r="E25" s="168"/>
       <c r="F25" s="168"/>
     </row>
-    <row r="26" ht="39" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:9" ht="39" x14ac:dyDescent="0.15">
       <c r="A26" s="183" t="s">
         <v>888</v>
       </c>
@@ -19512,11 +16307,6 @@
       </c>
       <c r="E26" s="168"/>
       <c r="F26" s="168"/>
-      <c r="J26" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found (Harrison 2025 prices only the 15 MPa pressurisation pump, 6.7 kW for 814 nozzles).</t>
-        </is>
-      </c>
     </row>
     <row r="27" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="170" t="s">
@@ -19692,359 +16482,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-  </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="70" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="48" customHeight="1">
-      <c r="A1" s="400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ADDED by precis/Reto, 2026-10-24 - NOT part of Tito's draft. Papers behind the literature notes, and the cells each supports.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Paper</t>
-        </is>
-      </c>
-      <c r="B3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DOI</t>
-        </is>
-      </c>
-      <c r="C3" s="399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cells it supports</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Harrison, Medcraft &amp; Harrison 2025, Environ. Sci.: Atmos., effervescent nozzle</t>
-        </is>
-      </c>
-      <c r="B4" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1039/D5EA00073D</t>
-        </is>
-      </c>
-      <c r="C4" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Technology Description!J8, J9, J10, J17, J23; 2. Cost Inputs!J13, J14; 5a!J12</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2026 (preprint), range of MCB radiative forcing across ESMs</t>
-        </is>
-      </c>
-      <c r="B5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/egusphere-2026-5460</t>
-        </is>
-      </c>
-      <c r="C5" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Technology Description!J10; 6a!N10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2026, J. Climate, forcing susceptibility (not checked)</t>
-        </is>
-      </c>
-      <c r="B6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1175/JCLI-D-25-0337.1</t>
-        </is>
-      </c>
-      <c r="C6" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!E7:E13 (source of the K per Tg/yr values); 6a!N10</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hernandez-Jaramillo, Kelaher &amp; Harrison 2025, plume dispersion review</t>
-        </is>
-      </c>
-      <c r="B7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3389/fmars.2025.1450175</t>
-        </is>
-      </c>
-      <c r="C7" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5a!J5; 6a!N32</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hernandez-Jaramillo et al. 2025, ERL, first outdoor MCB trial</t>
-        </is>
-      </c>
-      <c r="B8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1088/1748-9326/adccd7</t>
-        </is>
-      </c>
-      <c r="C8" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5a!J12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stjern et al. 2018, ACP, G4cdnc multi-model ensemble</t>
-        </is>
-      </c>
-      <c r="B9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-18-621-2018</t>
-        </is>
-      </c>
-      <c r="C9" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!N16</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Latham et al. 2012, Phil. Trans. R. Soc. A, Marine cloud brightening</t>
-        </is>
-      </c>
-      <c r="B10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1098/rsta.2012.0086</t>
-        </is>
-      </c>
-      <c r="C10" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Survey tab, section B</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hirasawa et al. 2023, GRL, regional MCB and tipping elements</t>
-        </is>
-      </c>
-      <c r="B11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1029/2023GL104314</t>
-        </is>
-      </c>
-      <c r="C11" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b!J19; 6c!J28</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Xie et al. 2022, ACP, solar geoengineering and the AMOC</t>
-        </is>
-      </c>
-      <c r="B12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.5194/acp-22-4581-2022</t>
-        </is>
-      </c>
-      <c r="C12" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b!J19</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tilmes et al. 2014, GRL, regional Arctic climate engineering</t>
-        </is>
-      </c>
-      <c r="B13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1002/2013GL058731</t>
-        </is>
-      </c>
-      <c r="C13" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Survey tab, section C</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">van Westen, Kliphuis &amp; Dijkstra 2024, Sci. Adv., AMOC early warning</t>
-        </is>
-      </c>
-      <c r="B14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1126/sciadv.adk1189</t>
-        </is>
-      </c>
-      <c r="C14" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Survey tab, section C</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Burke, Hsiang &amp; Miguel 2015, Nature, temperature and economic production</t>
-        </is>
-      </c>
-      <c r="B15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/nature15725</t>
-        </is>
-      </c>
-      <c r="C15" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!N44</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kotz, Levermann &amp; Wenz 2024, Nature (not checked)</t>
-        </is>
-      </c>
-      <c r="B16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.1038/s41586-024-07219-0</t>
-        </is>
-      </c>
-      <c r="C16" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!N45</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nordhaus 2016, NBER w22933, DICE-2016R (Projections and Uncertainties About Climate Change in an Era of Minimal Climate Policies)</t>
-        </is>
-      </c>
-      <c r="B17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3386/w22933</t>
-        </is>
-      </c>
-      <c r="C17" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!N43</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bilal &amp; Kanzig 2024, NBER w32450, The Macroeconomic Impact of Climate Change: Global vs. Local Temperature</t>
-        </is>
-      </c>
-      <c r="B18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://doi.org/10.3386/w32450</t>
-        </is>
-      </c>
-      <c r="C18" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6a!N45</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RRAP CS-06 and CS-07 final reports 2025; RRAP T14 (Harrison et al. 2019)</t>
-        </is>
-      </c>
-      <c r="B19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no DOI</t>
-        </is>
-      </c>
-      <c r="C19" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2. Cost Inputs!J40; 5a!J25</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PERILS AG industry loss announcements, SCS Cerry (20 Oct 2026) and Raphaela (19 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.perils.org/news</t>
-        </is>
-      </c>
-      <c r="C20" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6b!J19; 6c!J28; Summary tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gallagher Re Q3 2026 Natural Catastrophe and Climate Report, via Reinsurance News (21 Oct 2026)</t>
-        </is>
-      </c>
-      <c r="B21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.reinsurancene.ws/gallagher-re-reports-lowest-global-insured-catastrophe-losses-for-first-nine-months-since-2019</t>
-        </is>
-      </c>
-      <c r="C21" s="397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Survey tab, section F; Summary tab</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -20053,7 +16493,6 @@
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="69.5" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>
-    <col min="10" max="10" width="120" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -20081,7 +16520,7 @@
       <c r="D3" s="357"/>
       <c r="E3" s="357"/>
     </row>
-    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8"/>
       <c r="B4" s="8" t="s">
         <v>14</v>
@@ -20096,13 +16535,8 @@
       <c r="F4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>63</v>
       </c>
@@ -20119,13 +16553,8 @@
       <c r="F5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="J5" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>67</v>
       </c>
@@ -20142,13 +16571,8 @@
       <c r="F6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>71</v>
       </c>
@@ -20163,13 +16587,8 @@
       <c r="F7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J7" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>891</v>
       </c>
@@ -20184,11 +16603,6 @@
       </c>
       <c r="F8" s="2" t="s">
         <v>894</v>
-      </c>
-      <c r="J8" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20248,7 +16662,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="13" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>78</v>
       </c>
@@ -20265,13 +16679,8 @@
       </c>
       <c r="F13" s="354"/>
       <c r="G13" s="354"/>
-      <c r="J13" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: Harrison 2025 (https://doi.org/10.1039/D5EA00073D) needs 814 nozzles for 1e15 CCN/s; workbook 8,141 nozzles is exactly 10x, consistent with its 1e16/s.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>80</v>
       </c>
@@ -20287,11 +16696,6 @@
       </c>
       <c r="F14" t="s">
         <v>899</v>
-      </c>
-      <c r="J14" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: Harrison 2025 (https://doi.org/10.1039/D5EA00073D) gives 417.4 kW for 814 nozzles; workbook 4,168 kW is 10x, consistent.</t>
-        </is>
       </c>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20420,7 +16824,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>95</v>
       </c>
@@ -20438,11 +16842,6 @@
       </c>
       <c r="F25" s="2" t="s">
         <v>752</v>
-      </c>
-      <c r="J25" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No peer-reviewed value found; vessel spec sheets only.</t>
-        </is>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20519,7 +16918,7 @@
       </c>
       <c r="E30" s="27"/>
     </row>
-    <row r="31" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
         <v>105</v>
       </c>
@@ -20537,11 +16936,6 @@
       </c>
       <c r="F31" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="J31" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -20571,7 +16965,7 @@
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
     </row>
-    <row r="35" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
         <v>109</v>
       </c>
@@ -20587,11 +16981,6 @@
       </c>
       <c r="F35" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="J35" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
       </c>
     </row>
     <row r="36" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -20640,7 +17029,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="40" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
         <v>115</v>
       </c>
@@ -20670,13 +17059,8 @@
       <c r="I40" s="10" t="s">
         <v>903</v>
       </c>
-      <c r="J40" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: no published price for this nozzle. RRAP CS-07 final report 2025 gives MeeFog US$50/nozzle (report has no DOI). Workbook range $10-$1,000, selected $100 (H40 = 2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:9" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
         <v>116</v>
       </c>
@@ -20705,13 +17089,8 @@
       <c r="I41" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="J41" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found (used-equipment listing only).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="79" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:9" ht="79" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>118</v>
       </c>
@@ -20739,13 +17118,8 @@
       <c r="I42" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="J42" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; ballast-water systems are the only comparator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
         <v>120</v>
       </c>
@@ -20771,13 +17145,8 @@
       <c r="I43" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="J43" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found (workbook states nothing published exists).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:9" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
         <v>122</v>
       </c>
@@ -20798,11 +17167,6 @@
       </c>
       <c r="G44" s="9" t="s">
         <v>907</v>
-      </c>
-      <c r="J44" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No peer-reviewed value found (trade-press newbuild price basis).</t>
-        </is>
       </c>
     </row>
     <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20847,7 +17211,7 @@
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
         <v>128</v>
       </c>
@@ -20860,13 +17224,8 @@
       <c r="F49" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J49" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
         <v>130</v>
       </c>
@@ -20879,13 +17238,8 @@
       <c r="F50" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J50" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
         <v>131</v>
       </c>
@@ -20903,13 +17257,8 @@
       <c r="F51" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="J51" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
         <v>134</v>
       </c>
@@ -20921,11 +17270,6 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="J52" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
       </c>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -20959,7 +17303,7 @@
       </c>
       <c r="F55" s="8"/>
     </row>
-    <row r="56" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>908</v>
       </c>
@@ -20974,11 +17318,6 @@
       </c>
       <c r="E56" t="s">
         <v>832</v>
-      </c>
-      <c r="J56" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No literature value found; assumption.</t>
-        </is>
       </c>
     </row>
     <row r="57" spans="1:6" ht="30" x14ac:dyDescent="0.2">
@@ -26944,16 +23283,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="38" style="167" customWidth="1"/>
     <col min="2" max="3" width="18" style="167" customWidth="1"/>
     <col min="4" max="4" width="20" style="167" customWidth="1"/>
     <col min="5" max="5" width="50" style="167" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="167"/>
-    <col min="7" max="7" width="120" style="167" customWidth="1"/>
-    <col min="8" max="16384" width="8.6640625" style="167"/>
+    <col min="6" max="16384" width="8.6640625" style="167"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -26979,7 +23316,7 @@
       <c r="D4" s="366"/>
       <c r="E4" s="366"/>
     </row>
-    <row r="5" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A5" s="235" t="s">
         <v>764</v>
       </c>
@@ -26994,11 +23331,6 @@
       </c>
       <c r="E5" s="235" t="s">
         <v>766</v>
-      </c>
-      <c r="G5" s="403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFLICT: no '~$10B/yr' figure exists anywhere in this workbook (all tabs checked). Cost here is $21.4M/yr per dedicated vessel, $9.3M/yr per piggyback ship and $175B-$18T/yr for 1 K of global cooling (tabs 6b/6c). The ~$10B/yr figure in circulation traces only to a secondary summary of one review; no primary source found.</t>
-        </is>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -27092,7 +23424,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -27103,7 +23435,7 @@
     <col min="7" max="7" width="39.33203125" customWidth="1"/>
     <col min="8" max="8" width="55" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="120" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -27128,7 +23460,7 @@
       <c r="F2" s="368"/>
       <c r="G2" s="368"/>
     </row>
-    <row r="4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>57</v>
       </c>
@@ -27141,13 +23473,8 @@
       <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Literature note (added by precis/Reto, 2026-10-24; workbook values unchanged)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:8" ht="66.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>371</v>
       </c>
@@ -27165,11 +23492,6 @@
       <c r="G5" s="354"/>
       <c r="H5" s="2" t="s">
         <v>792</v>
-      </c>
-      <c r="J5" s="403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFLICT: no measured value; the plume review lists survival to cloud base as an open research gap (Hernandez-Jaramillo 2025, https://doi.org/10.3389/fmars.2025.1450175). The workbook 0.3 (range 0.1-0.5) has no literature backing.</t>
-        </is>
       </c>
     </row>
     <row r="6" spans="1:8" ht="79" customHeight="1" x14ac:dyDescent="0.2">
@@ -27277,7 +23599,7 @@
       <c r="F11" s="354"/>
       <c r="G11" s="354"/>
     </row>
-    <row r="12" ht="41.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="41.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>387</v>
       </c>
@@ -27295,11 +23617,6 @@
       <c r="G12" s="354"/>
       <c r="H12" s="2" t="s">
         <v>795</v>
-      </c>
-      <c r="J12" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lit: ~50 nm activates at 0.5% SS over the GBR (https://doi.org/10.1088/1748-9326/adccd7). CONFLICT: the nozzle's median dry size is 49.5 nm (Harrison 2025, https://doi.org/10.1039/D5EA00073D), so about half its particles sit at or below this threshold, while tab 1 uses 150 nm.</t>
-        </is>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" customHeight="1" x14ac:dyDescent="0.2">
@@ -27507,7 +23824,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="25" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>411</v>
       </c>
@@ -27525,11 +23842,6 @@
       <c r="G25" s="354"/>
       <c r="H25" s="2" t="s">
         <v>797</v>
-      </c>
-      <c r="J25" s="402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source report (RRAP T14, Harrison et al. 2019) has no DOI; value not checked.</t>
-        </is>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>